<commit_message>
Task 0 docs: PepsiCo client-styled summary workbook + branding module
- scripts/branding.py: reusable PepsiCo palette + generated brand icons
  (original stylized art, NOT official logos) with trademark disclaimer
- reframe Task0_Summary.xlsx to a PepsiCo engagement: portfolio in scope,
  PepsiCo-specific pain points (DSD, freshness, promos, NPI), M5-as-proxy note
- new 'PepsiCo Portfolio' sheet with 12 product icons + forecasting relevance
- add pillow to docs extra; icons in assets/brand/generated/
</commit_message>
<xml_diff>
--- a/docs/Task0_Summary.xlsx
+++ b/docs/Task0_Summary.xlsx
@@ -11,8 +11,9 @@
     <sheet name="Business Summary" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Developer Summary" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Concepts Covered" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Roadmap 0-18" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Task 0 Checklist" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="PepsiCo Portfolio" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Roadmap 0-18" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Task 0 Checklist" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -50,12 +51,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="002E75B6"/>
+        <fgColor rgb="0000307A"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="001F4E78"/>
+        <fgColor rgb="00004B93"/>
       </patternFill>
     </fill>
     <fill>
@@ -90,8 +91,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
@@ -178,6 +180,516 @@
     </indexedColors>
   </colors>
 </styleSheet>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>0</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="247650" cy="247650"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="1" name="Image 1" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
+</file>
+
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>0</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="247650" cy="247650"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="1" name="Image 1" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
+</file>
+
+<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>0</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="247650" cy="247650"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="1" name="Image 1" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
+</file>
+
+<file path=xl/drawings/drawing4.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>0</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="247650" cy="247650"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="1" name="Image 1" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
+</file>
+
+<file path=xl/drawings/drawing5.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>0</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="247650" cy="247650"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="1" name="Image 1" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>2</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="285750" cy="285750"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="2" name="Image 2" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId2"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>3</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="285750" cy="285750"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="3" name="Image 3" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId3"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>4</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="285750" cy="285750"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="4" name="Image 4" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId4"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>5</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="285750" cy="285750"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="5" name="Image 5" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId5"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>6</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="285750" cy="285750"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="6" name="Image 6" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId6"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>7</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="285750" cy="285750"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="7" name="Image 7" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId7"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>8</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="285750" cy="285750"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="8" name="Image 8" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId8"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>9</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="285750" cy="285750"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="9" name="Image 9" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId9"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>10</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="285750" cy="285750"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="10" name="Image 10" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId10"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>11</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="285750" cy="285750"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="11" name="Image 11" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId11"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>12</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="285750" cy="285750"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="12" name="Image 12" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId12"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>13</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="285750" cy="285750"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="13" name="Image 13" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId13"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
+</file>
+
+<file path=xl/drawings/drawing6.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>0</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="247650" cy="247650"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="1" name="Image 1" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
+</file>
+
+<file path=xl/drawings/drawing7.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>0</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="247650" cy="247650"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="1" name="Image 1" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -469,145 +981,171 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B11"/>
+  <dimension ref="A1:B13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="24" customWidth="1" min="1" max="1"/>
     <col width="95" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
-    <row r="1" ht="26" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>CPG Demand Forecasting — Project Overview</t>
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" s="1" t="n"/>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>PepsiCo Demand Forecasting — Project Overview</t>
         </is>
       </c>
     </row>
     <row r="2" ht="22" customHeight="1">
-      <c r="A2" s="2" t="inlineStr">
+      <c r="A2" s="3" t="inlineStr">
         <is>
           <t>Field</t>
         </is>
       </c>
-      <c r="B2" s="2" t="inlineStr">
+      <c r="B2" s="3" t="inlineStr">
         <is>
           <t>Detail</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="3" t="inlineStr">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>Client (illustrative)</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>PepsiCo, Inc. — global food &amp; beverage leader</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
         <is>
           <t>Project</t>
         </is>
       </c>
-      <c r="B3" s="3" t="inlineStr">
-        <is>
-          <t>End-to-end CPG SKU-level demand forecasting with time-series deep learning</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="3" t="inlineStr">
-        <is>
-          <t>Domain</t>
-        </is>
-      </c>
-      <c r="B4" s="3" t="inlineStr">
-        <is>
-          <t>Consumer Packaged Goods (CPG) / retail demand planning</t>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>End-to-end SKU-level demand forecasting with time-series deep learning</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="3" t="inlineStr">
+      <c r="A5" s="4" t="inlineStr">
         <is>
           <t>Purpose</t>
         </is>
       </c>
-      <c r="B5" s="3" t="inlineStr">
+      <c r="B5" s="4" t="inlineStr">
         <is>
           <t>Learning project: master the full deep-learning ladder end to end (data -&gt; deployment)</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="3" t="inlineStr">
-        <is>
-          <t>Dataset</t>
-        </is>
-      </c>
-      <c r="B6" s="3" t="inlineStr">
-        <is>
-          <t>M5 Forecasting - Accuracy (Walmart, via Kaggle): 42,840 hierarchical daily series</t>
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>Portfolio in scope</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>Beverages (Pepsi, Mtn Dew, Gatorade, Tropicana, Aquafina, 7UP) + Frito-Lay snacks (Lay's, Doritos, Cheetos, Ruffles) + Quaker foods</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="3" t="inlineStr">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>Data (proxy)</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>M5 Forecasting - Accuracy (Walmart, Kaggle) used as a realistic stand-in for PepsiCo's SKU x store x day sales; a real engagement would use PepsiCo shipment / POS / Nielsen data</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
         <is>
           <t>Forecast target</t>
         </is>
       </c>
-      <c r="B7" s="3" t="inlineStr">
+      <c r="B8" s="4" t="inlineStr">
         <is>
           <t>Units sold per SKU x store x day, 28-day horizon, with uncertainty intervals</t>
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="3" t="inlineStr">
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
         <is>
           <t>Primary metric</t>
         </is>
       </c>
-      <c r="B8" s="3" t="inlineStr">
-        <is>
-          <t>WRMSSE (M5 competition metric) + MAE / RMSE / pinball loss</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="3" t="inlineStr">
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>WRMSSE (M5 metric) + MAE / RMSE / pinball loss</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
         <is>
           <t>Repository</t>
         </is>
       </c>
-      <c r="B9" s="3" t="inlineStr">
+      <c r="B10" s="4" t="inlineStr">
         <is>
           <t>github.com/sudheerchowdary97/cpg-demand-forecasting (public, personal)</t>
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="3" t="inlineStr">
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
         <is>
           <t>Guardrails</t>
         </is>
       </c>
-      <c r="B10" s="3" t="inlineStr">
+      <c r="B11" s="4" t="inlineStr">
         <is>
           <t>No Apple ecosystem; heavy training on cloud GPU only; Mac used for light dev</t>
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="3" t="inlineStr">
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
         <is>
           <t>This workbook</t>
         </is>
       </c>
-      <c r="B11" s="3" t="inlineStr">
+      <c r="B12" s="4" t="inlineStr">
         <is>
           <t>Summary of Task 0 (Foundations &amp; Environment) — business + developer views</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>DISCLAIMER</t>
+        </is>
+      </c>
+      <c r="B13" s="4" t="inlineStr">
+        <is>
+          <t>Independent learning project; NOT affiliated with or endorsed by PepsiCo. Brand icons/colors are stylized, original representations — not official assets. All trademarks belong to their owners.</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:B1"/>
+    <mergeCell ref="B1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -617,196 +1155,232 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C11"/>
+  <dimension ref="A1:C13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
-    <col width="62" customWidth="1" min="2" max="2"/>
-    <col width="45" customWidth="1" min="3" max="3"/>
+    <col width="64" customWidth="1" min="2" max="2"/>
+    <col width="42" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
-    <row r="1" ht="26" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Business View — Objectives, Pain Points, Solution &amp; Pathway</t>
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" s="1" t="n"/>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>Business View — PepsiCo Objectives, Pain Points &amp; Solution</t>
         </is>
       </c>
     </row>
     <row r="2" ht="22" customHeight="1">
-      <c r="A2" s="2" t="inlineStr">
+      <c r="A2" s="3" t="inlineStr">
         <is>
           <t>Topic</t>
         </is>
       </c>
-      <c r="B2" s="2" t="inlineStr">
+      <c r="B2" s="3" t="inlineStr">
         <is>
           <t>Detail</t>
         </is>
       </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>Why it matters</t>
+      <c r="C2" s="3" t="inlineStr">
+        <is>
+          <t>Why it matters to PepsiCo</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="3" t="inlineStr">
+      <c r="A3" s="4" t="inlineStr">
         <is>
           <t>Business objective</t>
         </is>
       </c>
-      <c r="B3" s="3" t="inlineStr">
-        <is>
-          <t>Forecast product demand accurately at store level so the right stock is in the right place at the right time.</t>
-        </is>
-      </c>
-      <c r="C3" s="3" t="inlineStr">
-        <is>
-          <t>Directly drives revenue, availability, and working-capital efficiency.</t>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>Forecast demand accurately at store level so the right pack is on the right shelf at the right time across Pepsi, Frito-Lay and Quaker.</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>Directly drives net revenue, availability, and working capital.</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="3" t="inlineStr">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>Scale of the problem</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>~$91B annual net revenue, 20+ billion-dollar brands, products sold in 200+ countries/territories.</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>Tiny % accuracy gains compound into very large absolute value.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
         <is>
           <t>Pain point 1 — Stockouts</t>
         </is>
       </c>
-      <c r="B4" s="3" t="inlineStr">
-        <is>
-          <t>Running out of a product loses the sale and sends shoppers to competitors.</t>
-        </is>
-      </c>
-      <c r="C4" s="3" t="inlineStr">
-        <is>
-          <t>Lost sales are estimated at ~4% of revenue for typical retailers.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="3" t="inlineStr">
-        <is>
-          <t>Pain point 2 — Overstock</t>
-        </is>
-      </c>
-      <c r="B5" s="3" t="inlineStr">
-        <is>
-          <t>Too much stock leads to markdowns, spoilage (perishables), and cash tied up in inventory.</t>
-        </is>
-      </c>
-      <c r="C5" s="3" t="inlineStr">
-        <is>
-          <t>Waste and clearance directly erode margin.</t>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>Empty shelves lose the sale and push shoppers to competitor brands.</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>Lost sales estimated at ~4% of revenue for typical retailers.</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="3" t="inlineStr">
-        <is>
-          <t>Pain point 3 — Scale</t>
-        </is>
-      </c>
-      <c r="B6" s="3" t="inlineStr">
-        <is>
-          <t>Manual / spreadsheet forecasting cannot cover thousands of SKUs across many stores.</t>
-        </is>
-      </c>
-      <c r="C6" s="3" t="inlineStr">
-        <is>
-          <t>Human rules do not scale and are inconsistent.</t>
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>Pain point 2 — Waste / freshness</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>Frito-Lay snacks and chilled Tropicana are freshness-critical; overstock becomes stale/expired.</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>Waste and markdowns directly erode margin.</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="3" t="inlineStr">
-        <is>
-          <t>Pain point 4 — Demand spikes</t>
-        </is>
-      </c>
-      <c r="B7" s="3" t="inlineStr">
-        <is>
-          <t>Promotions, holidays, price changes, and local events cause swings classic methods miss.</t>
-        </is>
-      </c>
-      <c r="C7" s="3" t="inlineStr">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>Pain point 3 — DSD complexity</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>Direct-Store-Delivery routes must be stocked per store per day without over/under-loading trucks.</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>Route efficiency and service level depend on the forecast.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>Pain point 4 — Promotions &amp; events</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>Promos, price changes, holidays, sports events and heatwaves cause large demand swings.</t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="inlineStr">
         <is>
           <t>Missed spikes = stockouts; over-forecast = waste.</t>
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="3" t="inlineStr">
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>Pain point 5 — New product launches</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>Constant limited-time flavors and NPI have little/no history.</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="inlineStr">
+        <is>
+          <t>Cold-start forecasting is hard and high-stakes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
         <is>
           <t>Proposed solution</t>
         </is>
       </c>
-      <c r="B8" s="3" t="inlineStr">
-        <is>
-          <t>Deep-learning time-series models that forecast SKU x store x day demand with uncertainty, feeding replenishment, production, and promo planning.</t>
-        </is>
-      </c>
-      <c r="C8" s="3" t="inlineStr">
-        <is>
-          <t>Captures seasonality, promotions, and cross-series patterns automatically.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="3" t="inlineStr">
+      <c r="B10" s="4" t="inlineStr">
+        <is>
+          <t>Deep-learning time-series models forecasting SKU x store x day demand with uncertainty, feeding replenishment, DSD, production and promo planning.</t>
+        </is>
+      </c>
+      <c r="C10" s="4" t="inlineStr">
+        <is>
+          <t>Captures seasonality, promotions, weather and cross-brand patterns automatically.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
         <is>
           <t>Business value</t>
         </is>
       </c>
-      <c r="B9" s="3" t="inlineStr">
-        <is>
-          <t>Fewer stockouts, less waste, higher service levels, and data-driven, auditable planning decisions.</t>
-        </is>
-      </c>
-      <c r="C9" s="3" t="inlineStr">
+      <c r="B11" s="4" t="inlineStr">
+        <is>
+          <t>Fewer stockouts, less waste, higher service levels, tighter DSD, and data-driven, auditable planning.</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="inlineStr">
         <is>
           <t>Improves both top line (sales) and bottom line (margin).</t>
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="3" t="inlineStr">
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
         <is>
           <t>Pathway to impact</t>
         </is>
       </c>
-      <c r="B10" s="3" t="inlineStr">
-        <is>
-          <t>Forecasts -&gt; safety-stock &amp; replenishment orders -&gt; production plans -&gt; promo planning; served via a live API + planner dashboard.</t>
-        </is>
-      </c>
-      <c r="C10" s="3" t="inlineStr">
-        <is>
-          <t>Turns model output into day-to-day operational decisions.</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="3" t="inlineStr">
+      <c r="B12" s="4" t="inlineStr">
+        <is>
+          <t>Forecasts -&gt; safety stock &amp; replenishment -&gt; DSD route loads -&gt; production plans -&gt; promo planning; served via a live API + planner dashboard.</t>
+        </is>
+      </c>
+      <c r="C12" s="4" t="inlineStr">
+        <is>
+          <t>Turns model output into daily operational decisions.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
         <is>
           <t>Task 0 in business terms</t>
         </is>
       </c>
-      <c r="B11" s="3" t="inlineStr">
+      <c r="B13" s="4" t="inlineStr">
         <is>
           <t>Built a trustworthy, reproducible, vendor-neutral foundation before any modeling.</t>
         </is>
       </c>
-      <c r="C11" s="3" t="inlineStr">
-        <is>
-          <t>Ensures results are credible, auditable, and not locked to any vendor — reduces project risk.</t>
+      <c r="C13" s="4" t="inlineStr">
+        <is>
+          <t>Ensures results are credible and auditable — reduces project risk.</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="B1:C1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -816,7 +1390,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C13"/>
+  <dimension ref="A1:C14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -824,212 +1398,230 @@
     <col width="40" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
-    <row r="1" ht="26" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" s="1" t="n"/>
+      <c r="B1" s="2" t="inlineStr">
         <is>
           <t>Developer View — What Was Built in Task 0</t>
         </is>
       </c>
     </row>
     <row r="2" ht="22" customHeight="1">
-      <c r="A2" s="2" t="inlineStr">
+      <c r="A2" s="3" t="inlineStr">
         <is>
           <t>Area</t>
         </is>
       </c>
-      <c r="B2" s="2" t="inlineStr">
+      <c r="B2" s="3" t="inlineStr">
         <is>
           <t>What was done</t>
         </is>
       </c>
-      <c r="C2" s="2" t="inlineStr">
+      <c r="C2" s="3" t="inlineStr">
         <is>
           <t>Tool / Detail</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="3" t="inlineStr">
+      <c r="A3" s="4" t="inlineStr">
         <is>
           <t>Objective</t>
         </is>
       </c>
-      <c r="B3" s="3" t="inlineStr">
+      <c r="B3" s="4" t="inlineStr">
         <is>
           <t>Create a reproducible, industry-standard project skeleton before any DL code.</t>
         </is>
       </c>
-      <c r="C3" s="3" t="inlineStr">
+      <c r="C3" s="4" t="inlineStr">
         <is>
           <t>Foundations first</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="3" t="inlineStr">
+      <c r="A4" s="4" t="inlineStr">
         <is>
           <t>Package layout</t>
         </is>
       </c>
-      <c r="B4" s="3" t="inlineStr">
+      <c r="B4" s="4" t="inlineStr">
         <is>
           <t>src/ layout package 'cpg_forecast' installed as an editable package.</t>
         </is>
       </c>
-      <c r="C4" s="3" t="inlineStr">
+      <c r="C4" s="4" t="inlineStr">
         <is>
           <t>src/cpg_forecast/</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="3" t="inlineStr">
+      <c r="A5" s="4" t="inlineStr">
         <is>
           <t>Environment</t>
         </is>
       </c>
-      <c r="B5" s="3" t="inlineStr">
+      <c r="B5" s="4" t="inlineStr">
         <is>
           <t>Isolated virtual environment on Python 3.12 (3.14 removed — ML wheels unsupported).</t>
         </is>
       </c>
-      <c r="C5" s="3" t="inlineStr">
+      <c r="C5" s="4" t="inlineStr">
         <is>
           <t>Python 3.12.13, .venv</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="3" t="inlineStr">
+      <c r="A6" s="4" t="inlineStr">
         <is>
           <t>Dependencies</t>
         </is>
       </c>
-      <c r="B6" s="3" t="inlineStr">
+      <c r="B6" s="4" t="inlineStr">
         <is>
           <t>Single source of truth for deps + tool config; light core, DL deps deferred.</t>
         </is>
       </c>
-      <c r="C6" s="3" t="inlineStr">
+      <c r="C6" s="4" t="inlineStr">
         <is>
           <t>pyproject.toml (dev/docs extras)</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="3" t="inlineStr">
+      <c r="A7" s="4" t="inlineStr">
         <is>
           <t>Code quality</t>
         </is>
       </c>
-      <c r="B7" s="3" t="inlineStr">
+      <c r="B7" s="4" t="inlineStr">
         <is>
           <t>Auto-formatting + linting enforced automatically on every commit.</t>
         </is>
       </c>
-      <c r="C7" s="3" t="inlineStr">
+      <c r="C7" s="4" t="inlineStr">
         <is>
           <t>ruff + black via pre-commit</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="3" t="inlineStr">
+      <c r="A8" s="4" t="inlineStr">
         <is>
           <t>Testing</t>
         </is>
       </c>
-      <c r="B8" s="3" t="inlineStr">
+      <c r="B8" s="4" t="inlineStr">
         <is>
           <t>Smoke tests prove the package imports and toolchain runs green.</t>
         </is>
       </c>
-      <c r="C8" s="3" t="inlineStr">
+      <c r="C8" s="4" t="inlineStr">
         <is>
           <t>pytest (2 passed)</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="3" t="inlineStr">
+      <c r="A9" s="4" t="inlineStr">
         <is>
           <t>Automation</t>
         </is>
       </c>
-      <c r="B9" s="3" t="inlineStr">
+      <c r="B9" s="4" t="inlineStr">
         <is>
           <t>One-command workflows for setup, lint, format, test, summary.</t>
         </is>
       </c>
-      <c r="C9" s="3" t="inlineStr">
+      <c r="C9" s="4" t="inlineStr">
         <is>
           <t>Makefile</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="3" t="inlineStr">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>Branding</t>
+        </is>
+      </c>
+      <c r="B10" s="4" t="inlineStr">
+        <is>
+          <t>Reusable PepsiCo-styled icon/theme module powering all task workbooks.</t>
+        </is>
+      </c>
+      <c r="C10" s="4" t="inlineStr">
+        <is>
+          <t>scripts/branding.py (Pillow)</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
         <is>
           <t>Data / model hygiene</t>
         </is>
       </c>
-      <c r="B10" s="3" t="inlineStr">
+      <c r="B11" s="4" t="inlineStr">
         <is>
           <t>data/ and models/ git-ignored (DVC-tracked later); folders kept via .gitkeep.</t>
         </is>
       </c>
-      <c r="C10" s="3" t="inlineStr">
+      <c r="C11" s="4" t="inlineStr">
         <is>
           <t>.gitignore + DVC intent</t>
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="3" t="inlineStr">
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
         <is>
           <t>Version control</t>
         </is>
       </c>
-      <c r="B11" s="3" t="inlineStr">
+      <c r="B12" s="4" t="inlineStr">
         <is>
           <t>Standalone git repo, personal (non-Apple) identity, pushed to GitHub.</t>
         </is>
       </c>
-      <c r="C11" s="3" t="inlineStr">
+      <c r="C12" s="4" t="inlineStr">
         <is>
           <t>git + GitHub CLI</t>
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="3" t="inlineStr">
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
         <is>
           <t>Docs</t>
         </is>
       </c>
-      <c r="B12" s="3" t="inlineStr">
-        <is>
-          <t>README with full Task 0-18 roadmap; MIT license; this summary workbook.</t>
-        </is>
-      </c>
-      <c r="C12" s="3" t="inlineStr">
+      <c r="B13" s="4" t="inlineStr">
+        <is>
+          <t>README with full Task 0-18 roadmap; MIT license; this branded summary workbook.</t>
+        </is>
+      </c>
+      <c r="C13" s="4" t="inlineStr">
         <is>
           <t>README.md, LICENSE</t>
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="3" t="inlineStr">
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
         <is>
           <t>Deliberately NOT done</t>
         </is>
       </c>
-      <c r="B13" s="3" t="inlineStr">
+      <c r="B14" s="4" t="inlineStr">
         <is>
           <t>No neural networks yet — Task 0 is tooling only.</t>
         </is>
       </c>
-      <c r="C13" s="3" t="inlineStr">
+      <c r="C14" s="4" t="inlineStr">
         <is>
           <t>DL starts at Task 5</t>
         </is>
@@ -1037,9 +1629,10 @@
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="B1:C1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -1057,229 +1650,230 @@
     <col width="45" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
-    <row r="1" ht="26" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" s="1" t="n"/>
+      <c r="B1" s="2" t="inlineStr">
         <is>
           <t>Concepts &amp; Developer Skills Covered in Task 0</t>
         </is>
       </c>
     </row>
     <row r="2" ht="22" customHeight="1">
-      <c r="A2" s="2" t="inlineStr">
+      <c r="A2" s="3" t="inlineStr">
         <is>
           <t>Concept / Skill</t>
         </is>
       </c>
-      <c r="B2" s="2" t="inlineStr">
+      <c r="B2" s="3" t="inlineStr">
         <is>
           <t>What it is</t>
         </is>
       </c>
-      <c r="C2" s="2" t="inlineStr">
+      <c r="C2" s="3" t="inlineStr">
         <is>
           <t>Why it matters</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="3" t="inlineStr">
+      <c r="A3" s="4" t="inlineStr">
         <is>
           <t>src/ layout</t>
         </is>
       </c>
-      <c r="B3" s="3" t="inlineStr">
+      <c r="B3" s="4" t="inlineStr">
         <is>
           <t>Keeping importable code under src/ separate from tests/notebooks.</t>
         </is>
       </c>
-      <c r="C3" s="3" t="inlineStr">
+      <c r="C3" s="4" t="inlineStr">
         <is>
           <t>Prevents import bugs; industry-standard packaging.</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="3" t="inlineStr">
+      <c r="A4" s="4" t="inlineStr">
         <is>
           <t>Editable install</t>
         </is>
       </c>
-      <c r="B4" s="3" t="inlineStr">
+      <c r="B4" s="4" t="inlineStr">
         <is>
           <t>Installing the project with `pip install -e` so code changes apply instantly.</t>
         </is>
       </c>
-      <c r="C4" s="3" t="inlineStr">
+      <c r="C4" s="4" t="inlineStr">
         <is>
           <t>Real package imports without path hacks.</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="3" t="inlineStr">
+      <c r="A5" s="4" t="inlineStr">
         <is>
           <t>Virtual environment</t>
         </is>
       </c>
-      <c r="B5" s="3" t="inlineStr">
+      <c r="B5" s="4" t="inlineStr">
         <is>
           <t>An isolated Python env per project.</t>
         </is>
       </c>
-      <c r="C5" s="3" t="inlineStr">
+      <c r="C5" s="4" t="inlineStr">
         <is>
           <t>Reproducibility; no dependency clashes across projects.</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="3" t="inlineStr">
+      <c r="A6" s="4" t="inlineStr">
         <is>
           <t>pyproject.toml</t>
         </is>
       </c>
-      <c r="B6" s="3" t="inlineStr">
+      <c r="B6" s="4" t="inlineStr">
         <is>
           <t>Single file for dependencies + tool config (black, ruff, pytest).</t>
         </is>
       </c>
-      <c r="C6" s="3" t="inlineStr">
+      <c r="C6" s="4" t="inlineStr">
         <is>
           <t>One source of truth; modern Python standard.</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="3" t="inlineStr">
+      <c r="A7" s="4" t="inlineStr">
         <is>
           <t>Linting (ruff)</t>
         </is>
       </c>
-      <c r="B7" s="3" t="inlineStr">
+      <c r="B7" s="4" t="inlineStr">
         <is>
           <t>Static checks for errors, bugs, unused imports, import order.</t>
         </is>
       </c>
-      <c r="C7" s="3" t="inlineStr">
+      <c r="C7" s="4" t="inlineStr">
         <is>
           <t>Catches issues before runtime.</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="3" t="inlineStr">
+      <c r="A8" s="4" t="inlineStr">
         <is>
           <t>Formatting (black)</t>
         </is>
       </c>
-      <c r="B8" s="3" t="inlineStr">
+      <c r="B8" s="4" t="inlineStr">
         <is>
           <t>Deterministic, opinionated code formatting.</t>
         </is>
       </c>
-      <c r="C8" s="3" t="inlineStr">
+      <c r="C8" s="4" t="inlineStr">
         <is>
           <t>Consistent style; zero style debates.</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="3" t="inlineStr">
+      <c r="A9" s="4" t="inlineStr">
         <is>
           <t>pre-commit hooks</t>
         </is>
       </c>
-      <c r="B9" s="3" t="inlineStr">
+      <c r="B9" s="4" t="inlineStr">
         <is>
           <t>Checks that run automatically before each commit.</t>
         </is>
       </c>
-      <c r="C9" s="3" t="inlineStr">
+      <c r="C9" s="4" t="inlineStr">
         <is>
           <t>Bad code never enters git history.</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="3" t="inlineStr">
+      <c r="A10" s="4" t="inlineStr">
         <is>
           <t>Testing (pytest)</t>
         </is>
       </c>
-      <c r="B10" s="3" t="inlineStr">
+      <c r="B10" s="4" t="inlineStr">
         <is>
           <t>Automated tests, starting with smoke tests.</t>
         </is>
       </c>
-      <c r="C10" s="3" t="inlineStr">
+      <c r="C10" s="4" t="inlineStr">
         <is>
           <t>Confidence that the base works before building on it.</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="3" t="inlineStr">
+      <c r="A11" s="4" t="inlineStr">
         <is>
           <t>Makefile</t>
         </is>
       </c>
-      <c r="B11" s="3" t="inlineStr">
+      <c r="B11" s="4" t="inlineStr">
         <is>
           <t>Named shortcuts for common commands.</t>
         </is>
       </c>
-      <c r="C11" s="3" t="inlineStr">
+      <c r="C11" s="4" t="inlineStr">
         <is>
           <t>One-command, self-documenting workflows.</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="3" t="inlineStr">
+      <c r="A12" s="4" t="inlineStr">
         <is>
           <t>git + remote</t>
         </is>
       </c>
-      <c r="B12" s="3" t="inlineStr">
+      <c r="B12" s="4" t="inlineStr">
         <is>
           <t>Version control with a GitHub remote.</t>
         </is>
       </c>
-      <c r="C12" s="3" t="inlineStr">
+      <c r="C12" s="4" t="inlineStr">
         <is>
           <t>History, backup, collaboration, portfolio.</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="3" t="inlineStr">
+      <c r="A13" s="4" t="inlineStr">
         <is>
           <t>Data/model separation</t>
         </is>
       </c>
-      <c r="B13" s="3" t="inlineStr">
+      <c r="B13" s="4" t="inlineStr">
         <is>
           <t>Keeping large data &amp; artifacts out of git (DVC later).</t>
         </is>
       </c>
-      <c r="C13" s="3" t="inlineStr">
+      <c r="C13" s="4" t="inlineStr">
         <is>
           <t>Keeps repo small; data versioned properly.</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="3" t="inlineStr">
+      <c r="A14" s="4" t="inlineStr">
         <is>
           <t>Reproducibility</t>
         </is>
       </c>
-      <c r="B14" s="3" t="inlineStr">
+      <c r="B14" s="4" t="inlineStr">
         <is>
           <t>Pinned Python + pinned deps + scripted setup.</t>
         </is>
       </c>
-      <c r="C14" s="3" t="inlineStr">
+      <c r="C14" s="4" t="inlineStr">
         <is>
           <t>Anyone can rebuild the exact environment.</t>
         </is>
@@ -1287,13 +1881,284 @@
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="B1:C1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D14"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="3" max="3"/>
+    <col width="60" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" s="1" t="n"/>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>PepsiCo Portfolio in Scope — Brands &amp; Forecasting Relevance</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="22" customHeight="1">
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t>Icon</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>Brand</t>
+        </is>
+      </c>
+      <c r="C2" s="3" t="inlineStr">
+        <is>
+          <t>Category</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="inlineStr">
+        <is>
+          <t>Forecasting relevance</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="34" customHeight="1">
+      <c r="A3" s="4" t="inlineStr"/>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>🥤 Pepsi</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>Carbonated soft drinks</t>
+        </is>
+      </c>
+      <c r="D3" s="4" t="inlineStr">
+        <is>
+          <t>Top-volume CSD; strong summer &amp; holiday peaks, heavy promo lift.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="34" customHeight="1">
+      <c r="A4" s="4" t="inlineStr"/>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>🏔 Mountain Dew</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>Carbonated soft drinks</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="inlineStr">
+        <is>
+          <t>Youth-skewed CSD; limited-time flavors drive sharp launch spikes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="34" customHeight="1">
+      <c r="A5" s="4" t="inlineStr"/>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>⚡ Gatorade</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>Sports drinks</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>Sports/heat-driven; demand tracks temperature and sports seasons.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="34" customHeight="1">
+      <c r="A6" s="4" t="inlineStr"/>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>🍊 Tropicana</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>Chilled juices</t>
+        </is>
+      </c>
+      <c r="D6" s="4" t="inlineStr">
+        <is>
+          <t>Chilled juice; short shelf life, breakfast + winter-cold seasonality.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="34" customHeight="1">
+      <c r="A7" s="4" t="inlineStr"/>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>💧 Aquafina</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>Bottled water</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t>Water; strong summer and heatwave sensitivity.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="34" customHeight="1">
+      <c r="A8" s="4" t="inlineStr"/>
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>🥤 7UP</t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="inlineStr">
+        <is>
+          <t>Carbonated soft drinks</t>
+        </is>
+      </c>
+      <c r="D8" s="4" t="inlineStr">
+        <is>
+          <t>CSD; festive/holiday and mixer demand.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="34" customHeight="1">
+      <c r="A9" s="4" t="inlineStr"/>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>🥔 Lay's</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="inlineStr">
+        <is>
+          <t>Salty snacks (Frito-Lay)</t>
+        </is>
+      </c>
+      <c r="D9" s="4" t="inlineStr">
+        <is>
+          <t>DSD salty snack; freshness-critical, very high promo frequency.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="34" customHeight="1">
+      <c r="A10" s="4" t="inlineStr"/>
+      <c r="B10" s="4" t="inlineStr">
+        <is>
+          <t>🔺 Doritos</t>
+        </is>
+      </c>
+      <c r="C10" s="4" t="inlineStr">
+        <is>
+          <t>Salty snacks (Frito-Lay)</t>
+        </is>
+      </c>
+      <c r="D10" s="4" t="inlineStr">
+        <is>
+          <t>Snack; big-game/event and limited-edition spikes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="34" customHeight="1">
+      <c r="A11" s="4" t="inlineStr"/>
+      <c r="B11" s="4" t="inlineStr">
+        <is>
+          <t>🐆 Cheetos</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="inlineStr">
+        <is>
+          <t>Salty snacks (Frito-Lay)</t>
+        </is>
+      </c>
+      <c r="D11" s="4" t="inlineStr">
+        <is>
+          <t>Snack; steady base with promo-driven lift.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="34" customHeight="1">
+      <c r="A12" s="4" t="inlineStr"/>
+      <c r="B12" s="4" t="inlineStr">
+        <is>
+          <t>🥔 Ruffles</t>
+        </is>
+      </c>
+      <c r="C12" s="4" t="inlineStr">
+        <is>
+          <t>Salty snacks (Frito-Lay)</t>
+        </is>
+      </c>
+      <c r="D12" s="4" t="inlineStr">
+        <is>
+          <t>Snack; party/occasion and promo sensitive.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="34" customHeight="1">
+      <c r="A13" s="4" t="inlineStr"/>
+      <c r="B13" s="4" t="inlineStr">
+        <is>
+          <t>🥣 Quaker</t>
+        </is>
+      </c>
+      <c r="C13" s="4" t="inlineStr">
+        <is>
+          <t>Foods / oats</t>
+        </is>
+      </c>
+      <c r="D13" s="4" t="inlineStr">
+        <is>
+          <t>Ambient breakfast; longer shelf life, winter skew.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="34" customHeight="1">
+      <c r="A14" s="4" t="inlineStr"/>
+      <c r="B14" s="4" t="inlineStr">
+        <is>
+          <t>⚡ Rockstar</t>
+        </is>
+      </c>
+      <c r="C14" s="4" t="inlineStr">
+        <is>
+          <t>Energy drinks</t>
+        </is>
+      </c>
+      <c r="D14" s="4" t="inlineStr">
+        <is>
+          <t>Energy; convenience-channel, weekday skew.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="B1:D1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1309,548 +2174,549 @@
     <col width="12" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
-    <row r="1" ht="26" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" s="1" t="n"/>
+      <c r="B1" s="2" t="inlineStr">
         <is>
           <t>Full Roadmap — Task 0 to 18</t>
         </is>
       </c>
     </row>
     <row r="2" ht="22" customHeight="1">
-      <c r="A2" s="2" t="inlineStr">
+      <c r="A2" s="3" t="inlineStr">
         <is>
           <t>Task</t>
         </is>
       </c>
-      <c r="B2" s="2" t="inlineStr">
+      <c r="B2" s="3" t="inlineStr">
         <is>
           <t>Name</t>
         </is>
       </c>
-      <c r="C2" s="2" t="inlineStr">
+      <c r="C2" s="3" t="inlineStr">
         <is>
           <t>Core DL concept</t>
         </is>
       </c>
-      <c r="D2" s="2" t="inlineStr">
+      <c r="D2" s="3" t="inlineStr">
         <is>
           <t>Engineering skill</t>
         </is>
       </c>
-      <c r="E2" s="2" t="inlineStr">
+      <c r="E2" s="3" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="4" t="inlineStr">
+      <c r="A3" s="5" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="B3" s="4" t="inlineStr">
+      <c r="B3" s="5" t="inlineStr">
         <is>
           <t>Foundations &amp; environment</t>
         </is>
       </c>
-      <c r="C3" s="4" t="inlineStr">
+      <c r="C3" s="5" t="inlineStr">
         <is>
           <t>— (tooling)</t>
         </is>
       </c>
-      <c r="D3" s="4" t="inlineStr">
+      <c r="D3" s="5" t="inlineStr">
         <is>
           <t>repo layout, venv, linting, tests</t>
         </is>
       </c>
-      <c r="E3" s="4" t="inlineStr">
+      <c r="E3" s="5" t="inlineStr">
         <is>
           <t>Done ✅</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="3" t="inlineStr">
+      <c r="A4" s="4" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="B4" s="3" t="inlineStr">
+      <c r="B4" s="4" t="inlineStr">
         <is>
           <t>Problem framing &amp; data (DVC)</t>
         </is>
       </c>
-      <c r="C4" s="3" t="inlineStr">
+      <c r="C4" s="4" t="inlineStr">
         <is>
           <t>forecast task formulation</t>
         </is>
       </c>
-      <c r="D4" s="3" t="inlineStr">
+      <c r="D4" s="4" t="inlineStr">
         <is>
           <t>data versioning</t>
         </is>
       </c>
-      <c r="E4" s="3" t="inlineStr">
+      <c r="E4" s="4" t="inlineStr">
         <is>
           <t>Next</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="3" t="inlineStr">
+      <c r="A5" s="4" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="B5" s="3" t="inlineStr">
+      <c r="B5" s="4" t="inlineStr">
         <is>
           <t>EDA &amp; time-series understanding</t>
         </is>
       </c>
-      <c r="C5" s="3" t="inlineStr">
+      <c r="C5" s="4" t="inlineStr">
         <is>
           <t>seasonality, stationarity</t>
         </is>
       </c>
-      <c r="D5" s="3" t="inlineStr">
+      <c r="D5" s="4" t="inlineStr">
         <is>
           <t>reproducible notebooks</t>
         </is>
       </c>
-      <c r="E5" s="3" t="inlineStr">
+      <c r="E5" s="4" t="inlineStr">
         <is>
           <t>Planned</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="3" t="inlineStr">
+      <c r="A6" s="4" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="B6" s="3" t="inlineStr">
+      <c r="B6" s="4" t="inlineStr">
         <is>
           <t>Data pipeline &amp; feature engineering</t>
         </is>
       </c>
-      <c r="C6" s="3" t="inlineStr">
+      <c r="C6" s="4" t="inlineStr">
         <is>
           <t>windowing, embeddings</t>
         </is>
       </c>
-      <c r="D6" s="3" t="inlineStr">
+      <c r="D6" s="4" t="inlineStr">
         <is>
           <t>leakage-free ETL as code</t>
         </is>
       </c>
-      <c r="E6" s="3" t="inlineStr">
+      <c r="E6" s="4" t="inlineStr">
         <is>
           <t>Planned</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="3" t="inlineStr">
+      <c r="A7" s="4" t="inlineStr">
         <is>
           <t>4</t>
         </is>
       </c>
-      <c r="B7" s="3" t="inlineStr">
+      <c r="B7" s="4" t="inlineStr">
         <is>
           <t>Classical baselines &amp; eval harness</t>
         </is>
       </c>
-      <c r="C7" s="3" t="inlineStr">
+      <c r="C7" s="4" t="inlineStr">
         <is>
           <t>why baselines matter</t>
         </is>
       </c>
-      <c r="D7" s="3" t="inlineStr">
+      <c r="D7" s="4" t="inlineStr">
         <is>
           <t>WRMSSE, backtesting, tracking</t>
         </is>
       </c>
-      <c r="E7" s="3" t="inlineStr">
+      <c r="E7" s="4" t="inlineStr">
         <is>
           <t>Planned</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="3" t="inlineStr">
+      <c r="A8" s="4" t="inlineStr">
         <is>
           <t>5</t>
         </is>
       </c>
-      <c r="B8" s="3" t="inlineStr">
+      <c r="B8" s="4" t="inlineStr">
         <is>
           <t>MLP forecaster</t>
         </is>
       </c>
-      <c r="C8" s="3" t="inlineStr">
+      <c r="C8" s="4" t="inlineStr">
         <is>
           <t>MLPs, backprop, regularization</t>
         </is>
       </c>
-      <c r="D8" s="3" t="inlineStr">
+      <c r="D8" s="4" t="inlineStr">
         <is>
           <t>Lightning training loop</t>
         </is>
       </c>
-      <c r="E8" s="3" t="inlineStr">
+      <c r="E8" s="4" t="inlineStr">
         <is>
           <t>Planned</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="3" t="inlineStr">
+      <c r="A9" s="4" t="inlineStr">
         <is>
           <t>6</t>
         </is>
       </c>
-      <c r="B9" s="3" t="inlineStr">
+      <c r="B9" s="4" t="inlineStr">
         <is>
           <t>RNN -&gt; LSTM -&gt; GRU</t>
         </is>
       </c>
-      <c r="C9" s="3" t="inlineStr">
+      <c r="C9" s="4" t="inlineStr">
         <is>
           <t>recurrence, gating</t>
         </is>
       </c>
-      <c r="D9" s="3" t="inlineStr">
+      <c r="D9" s="4" t="inlineStr">
         <is>
           <t>GPU training discipline</t>
         </is>
       </c>
-      <c r="E9" s="3" t="inlineStr">
+      <c r="E9" s="4" t="inlineStr">
         <is>
           <t>Planned</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="3" t="inlineStr">
+      <c r="A10" s="4" t="inlineStr">
         <is>
           <t>7</t>
         </is>
       </c>
-      <c r="B10" s="3" t="inlineStr">
+      <c r="B10" s="4" t="inlineStr">
         <is>
           <t>Seq2Seq + Attention</t>
         </is>
       </c>
-      <c r="C10" s="3" t="inlineStr">
+      <c r="C10" s="4" t="inlineStr">
         <is>
           <t>attention, multi-horizon</t>
         </is>
       </c>
-      <c r="D10" s="3" t="inlineStr">
+      <c r="D10" s="4" t="inlineStr">
         <is>
           <t>attention visualization</t>
         </is>
       </c>
-      <c r="E10" s="3" t="inlineStr">
+      <c r="E10" s="4" t="inlineStr">
         <is>
           <t>Planned</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="3" t="inlineStr">
+      <c r="A11" s="4" t="inlineStr">
         <is>
           <t>8</t>
         </is>
       </c>
-      <c r="B11" s="3" t="inlineStr">
+      <c r="B11" s="4" t="inlineStr">
         <is>
           <t>Temporal Conv Nets (TCN)</t>
         </is>
       </c>
-      <c r="C11" s="3" t="inlineStr">
+      <c r="C11" s="4" t="inlineStr">
         <is>
           <t>dilated causal convolution</t>
         </is>
       </c>
-      <c r="D11" s="3" t="inlineStr">
+      <c r="D11" s="4" t="inlineStr">
         <is>
           <t>architecture ablation</t>
         </is>
       </c>
-      <c r="E11" s="3" t="inlineStr">
+      <c r="E11" s="4" t="inlineStr">
         <is>
           <t>Planned</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="3" t="inlineStr">
+      <c r="A12" s="4" t="inlineStr">
         <is>
           <t>9</t>
         </is>
       </c>
-      <c r="B12" s="3" t="inlineStr">
+      <c r="B12" s="4" t="inlineStr">
         <is>
           <t>Transformer / TFT</t>
         </is>
       </c>
-      <c r="C12" s="3" t="inlineStr">
+      <c r="C12" s="4" t="inlineStr">
         <is>
           <t>self-attention, interpretability</t>
         </is>
       </c>
-      <c r="D12" s="3" t="inlineStr">
+      <c r="D12" s="4" t="inlineStr">
         <is>
           <t>large-model training</t>
         </is>
       </c>
-      <c r="E12" s="3" t="inlineStr">
+      <c r="E12" s="4" t="inlineStr">
         <is>
           <t>Planned</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="3" t="inlineStr">
+      <c r="A13" s="4" t="inlineStr">
         <is>
           <t>10</t>
         </is>
       </c>
-      <c r="B13" s="3" t="inlineStr">
+      <c r="B13" s="4" t="inlineStr">
         <is>
           <t>Probabilistic (DeepAR / N-BEATS)</t>
         </is>
       </c>
-      <c r="C13" s="3" t="inlineStr">
+      <c r="C13" s="4" t="inlineStr">
         <is>
           <t>uncertainty, intermittency</t>
         </is>
       </c>
-      <c r="D13" s="3" t="inlineStr">
+      <c r="D13" s="4" t="inlineStr">
         <is>
           <t>calibration</t>
         </is>
       </c>
-      <c r="E13" s="3" t="inlineStr">
+      <c r="E13" s="4" t="inlineStr">
         <is>
           <t>Planned</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="3" t="inlineStr">
+      <c r="A14" s="4" t="inlineStr">
         <is>
           <t>11</t>
         </is>
       </c>
-      <c r="B14" s="3" t="inlineStr">
+      <c r="B14" s="4" t="inlineStr">
         <is>
           <t>Tracking, HPO &amp; model selection</t>
         </is>
       </c>
-      <c r="C14" s="3" t="inlineStr">
+      <c r="C14" s="4" t="inlineStr">
         <is>
           <t>HPO, bias/variance</t>
         </is>
       </c>
-      <c r="D14" s="3" t="inlineStr">
+      <c r="D14" s="4" t="inlineStr">
         <is>
           <t>Optuna + MLflow</t>
         </is>
       </c>
-      <c r="E14" s="3" t="inlineStr">
+      <c r="E14" s="4" t="inlineStr">
         <is>
           <t>Planned</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="3" t="inlineStr">
+      <c r="A15" s="4" t="inlineStr">
         <is>
           <t>12</t>
         </is>
       </c>
-      <c r="B15" s="3" t="inlineStr">
+      <c r="B15" s="4" t="inlineStr">
         <is>
           <t>Cloud full-scale training</t>
         </is>
       </c>
-      <c r="C15" s="3" t="inlineStr">
+      <c r="C15" s="4" t="inlineStr">
         <is>
           <t>mixed precision, checkpointing</t>
         </is>
       </c>
-      <c r="D15" s="3" t="inlineStr">
+      <c r="D15" s="4" t="inlineStr">
         <is>
           <t>training-as-code</t>
         </is>
       </c>
-      <c r="E15" s="3" t="inlineStr">
+      <c r="E15" s="4" t="inlineStr">
         <is>
           <t>Planned</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="3" t="inlineStr">
+      <c r="A16" s="4" t="inlineStr">
         <is>
           <t>13</t>
         </is>
       </c>
-      <c r="B16" s="3" t="inlineStr">
+      <c r="B16" s="4" t="inlineStr">
         <is>
           <t>Export &amp; optimize (ONNX / quantize)</t>
         </is>
       </c>
-      <c r="C16" s="3" t="inlineStr">
+      <c r="C16" s="4" t="inlineStr">
         <is>
           <t>graph export, quantization</t>
         </is>
       </c>
-      <c r="D16" s="3" t="inlineStr">
+      <c r="D16" s="4" t="inlineStr">
         <is>
           <t>perf benchmarking</t>
         </is>
       </c>
-      <c r="E16" s="3" t="inlineStr">
+      <c r="E16" s="4" t="inlineStr">
         <is>
           <t>Planned</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="3" t="inlineStr">
+      <c r="A17" s="4" t="inlineStr">
         <is>
           <t>14</t>
         </is>
       </c>
-      <c r="B17" s="3" t="inlineStr">
+      <c r="B17" s="4" t="inlineStr">
         <is>
           <t>Serving API (FastAPI + Docker)</t>
         </is>
       </c>
-      <c r="C17" s="3" t="inlineStr">
+      <c r="C17" s="4" t="inlineStr">
         <is>
           <t>inference-time preprocessing</t>
         </is>
       </c>
-      <c r="D17" s="3" t="inlineStr">
+      <c r="D17" s="4" t="inlineStr">
         <is>
           <t>API design, containers</t>
         </is>
       </c>
-      <c r="E17" s="3" t="inlineStr">
+      <c r="E17" s="4" t="inlineStr">
         <is>
           <t>Planned</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="3" t="inlineStr">
+      <c r="A18" s="4" t="inlineStr">
         <is>
           <t>15</t>
         </is>
       </c>
-      <c r="B18" s="3" t="inlineStr">
+      <c r="B18" s="4" t="inlineStr">
         <is>
           <t>Cloud deploy + CI/CD</t>
         </is>
       </c>
-      <c r="C18" s="3" t="inlineStr">
+      <c r="C18" s="4" t="inlineStr">
         <is>
           <t>production readiness</t>
         </is>
       </c>
-      <c r="D18" s="3" t="inlineStr">
+      <c r="D18" s="4" t="inlineStr">
         <is>
           <t>Cloud Run/Render, GitHub Actions</t>
         </is>
       </c>
-      <c r="E18" s="3" t="inlineStr">
+      <c r="E18" s="4" t="inlineStr">
         <is>
           <t>Planned</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="3" t="inlineStr">
+      <c r="A19" s="4" t="inlineStr">
         <is>
           <t>16</t>
         </is>
       </c>
-      <c r="B19" s="3" t="inlineStr">
+      <c r="B19" s="4" t="inlineStr">
         <is>
           <t>Monitoring, drift &amp; retraining</t>
         </is>
       </c>
-      <c r="C19" s="3" t="inlineStr">
+      <c r="C19" s="4" t="inlineStr">
         <is>
           <t>distribution shift</t>
         </is>
       </c>
-      <c r="D19" s="3" t="inlineStr">
+      <c r="D19" s="4" t="inlineStr">
         <is>
           <t>observability</t>
         </is>
       </c>
-      <c r="E19" s="3" t="inlineStr">
+      <c r="E19" s="4" t="inlineStr">
         <is>
           <t>Planned</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="3" t="inlineStr">
+      <c r="A20" s="4" t="inlineStr">
         <is>
           <t>17</t>
         </is>
       </c>
-      <c r="B20" s="3" t="inlineStr">
+      <c r="B20" s="4" t="inlineStr">
         <is>
           <t>Demo app + LLM insight layer</t>
         </is>
       </c>
-      <c r="C20" s="3" t="inlineStr">
+      <c r="C20" s="4" t="inlineStr">
         <is>
           <t>communicating uncertainty</t>
         </is>
       </c>
-      <c r="D20" s="3" t="inlineStr">
+      <c r="D20" s="4" t="inlineStr">
         <is>
           <t>Streamlit, prompt design</t>
         </is>
       </c>
-      <c r="E20" s="3" t="inlineStr">
+      <c r="E20" s="4" t="inlineStr">
         <is>
           <t>Planned</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="3" t="inlineStr">
+      <c r="A21" s="4" t="inlineStr">
         <is>
           <t>18</t>
         </is>
       </c>
-      <c r="B21" s="3" t="inlineStr">
+      <c r="B21" s="4" t="inlineStr">
         <is>
           <t>Docs, presentation &amp; portfolio</t>
         </is>
       </c>
-      <c r="C21" s="3" t="inlineStr">
+      <c r="C21" s="4" t="inlineStr">
         <is>
           <t>synthesis</t>
         </is>
       </c>
-      <c r="D21" s="3" t="inlineStr">
+      <c r="D21" s="4" t="inlineStr">
         <is>
           <t>technical writing, Keynote-HTML</t>
         </is>
       </c>
-      <c r="E21" s="3" t="inlineStr">
+      <c r="E21" s="4" t="inlineStr">
         <is>
           <t>Planned</t>
         </is>
@@ -1858,171 +2724,185 @@
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:E1"/>
+    <mergeCell ref="B1:E1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B13"/>
+  <dimension ref="A1:B14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="65" customWidth="1" min="1" max="1"/>
     <col width="14" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
-    <row r="1" ht="26" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" s="1" t="n"/>
+      <c r="B1" s="2" t="inlineStr">
         <is>
           <t>Task 0 — Deliverables Checklist</t>
         </is>
       </c>
     </row>
     <row r="2" ht="22" customHeight="1">
-      <c r="A2" s="2" t="inlineStr">
+      <c r="A2" s="3" t="inlineStr">
         <is>
           <t>Deliverable</t>
         </is>
       </c>
-      <c r="B2" s="2" t="inlineStr">
+      <c r="B2" s="3" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="4" t="inlineStr">
+      <c r="A3" s="5" t="inlineStr">
         <is>
           <t>src/ layout package (cpg_forecast) installed editable</t>
         </is>
       </c>
-      <c r="B3" s="4" t="inlineStr">
+      <c r="B3" s="5" t="inlineStr">
         <is>
           <t>Done ✅</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="4" t="inlineStr">
+      <c r="A4" s="5" t="inlineStr">
         <is>
           <t>Python 3.12 virtual environment</t>
         </is>
       </c>
-      <c r="B4" s="4" t="inlineStr">
+      <c r="B4" s="5" t="inlineStr">
         <is>
           <t>Done ✅</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="4" t="inlineStr">
+      <c r="A5" s="5" t="inlineStr">
         <is>
           <t>pyproject.toml with dev + docs extras</t>
         </is>
       </c>
-      <c r="B5" s="4" t="inlineStr">
+      <c r="B5" s="5" t="inlineStr">
         <is>
           <t>Done ✅</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="4" t="inlineStr">
+      <c r="A6" s="5" t="inlineStr">
         <is>
           <t>ruff + black wired via pre-commit</t>
         </is>
       </c>
-      <c r="B6" s="4" t="inlineStr">
+      <c r="B6" s="5" t="inlineStr">
         <is>
           <t>Done ✅</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="4" t="inlineStr">
+      <c r="A7" s="5" t="inlineStr">
         <is>
           <t>Passing smoke tests (pytest)</t>
         </is>
       </c>
-      <c r="B7" s="4" t="inlineStr">
+      <c r="B7" s="5" t="inlineStr">
         <is>
           <t>Done ✅</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="4" t="inlineStr">
+      <c r="A8" s="5" t="inlineStr">
         <is>
           <t>Makefile (setup/lint/format/test/summary)</t>
         </is>
       </c>
-      <c r="B8" s="4" t="inlineStr">
+      <c r="B8" s="5" t="inlineStr">
         <is>
           <t>Done ✅</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="4" t="inlineStr">
+      <c r="A9" s="5" t="inlineStr">
         <is>
           <t>.gitignore + DVC-ready data/model folders</t>
         </is>
       </c>
-      <c r="B9" s="4" t="inlineStr">
+      <c r="B9" s="5" t="inlineStr">
         <is>
           <t>Done ✅</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="4" t="inlineStr">
+      <c r="A10" s="5" t="inlineStr">
         <is>
           <t>README with full roadmap + MIT LICENSE</t>
         </is>
       </c>
-      <c r="B10" s="4" t="inlineStr">
+      <c r="B10" s="5" t="inlineStr">
         <is>
           <t>Done ✅</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="4" t="inlineStr">
+      <c r="A11" s="5" t="inlineStr">
         <is>
           <t>Personal (non-Apple) git identity</t>
         </is>
       </c>
-      <c r="B11" s="4" t="inlineStr">
+      <c r="B11" s="5" t="inlineStr">
         <is>
           <t>Done ✅</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="4" t="inlineStr">
+      <c r="A12" s="5" t="inlineStr">
         <is>
           <t>Repo created &amp; pushed to personal GitHub</t>
         </is>
       </c>
-      <c r="B12" s="4" t="inlineStr">
+      <c r="B12" s="5" t="inlineStr">
         <is>
           <t>Done ✅</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="4" t="inlineStr">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>PepsiCo-styled branding module (icons/theme)</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="inlineStr">
+        <is>
+          <t>Done ✅</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
         <is>
           <t>Business + developer summary workbook (this file)</t>
         </is>
       </c>
-      <c r="B13" s="4" t="inlineStr">
+      <c r="B14" s="5" t="inlineStr">
         <is>
           <t>Done ✅</t>
         </is>
@@ -2030,8 +2910,9 @@
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:B1"/>
+    <mergeCell ref="B1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Task 0 docs: scale workbook to multi-geo, all-brands PepsiCo scope
- use real PepsiCo logo (user-supplied) on all sheet title bars
- branding.py: GEOS (UK/AU/IN/PK) + 20-brand master data (kind, colors,
  market coverage); generate icons for every brand; JPEG-compress infographic
- new sheets: Global Brand Matrix (brands x market) and Global Portfolio Map
  (embedded infographic); Brand Portfolio expanded with icons + markets column
- Overview/Business reframed for global scaling (one model, geo/brand
  embeddings, hemisphere seasonality, local festivals, cold-start)
- gitignore raw brand source drops; commit optimized derived assets
</commit_message>
<xml_diff>
--- a/docs/Task0_Summary.xlsx
+++ b/docs/Task0_Summary.xlsx
@@ -11,9 +11,11 @@
     <sheet name="Business Summary" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Developer Summary" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Concepts Covered" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="PepsiCo Portfolio" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Roadmap 0-18" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Task 0 Checklist" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Global Brand Matrix" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Brand Portfolio" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Global Portfolio Map" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Roadmap 0-18" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Task 0 Checklist" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -23,7 +25,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="3">
+  <fonts count="5">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -33,13 +35,22 @@
     </font>
     <font>
       <b val="1"/>
-      <color rgb="00FFFFFF"/>
+      <color rgb="00004B93"/>
       <sz val="14"/>
     </font>
     <font>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
       <sz val="11"/>
+    </font>
+    <font>
+      <i val="1"/>
+      <color rgb="00004B93"/>
+    </font>
+    <font>
+      <i val="1"/>
+      <color rgb="00808080"/>
+      <sz val="9"/>
     </font>
   </fonts>
   <fills count="5">
@@ -51,7 +62,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="0000307A"/>
+        <fgColor rgb="00FFFFFF"/>
       </patternFill>
     </fill>
     <fill>
@@ -91,7 +102,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -103,6 +114,10 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -191,7 +206,7 @@
       <row>0</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="247650" cy="247650"/>
+    <ext cx="495300" cy="285750"/>
     <pic>
       <nvPicPr>
         <cNvPr id="1" name="Image 1" descr="Picture"/>
@@ -221,7 +236,7 @@
       <row>0</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="247650" cy="247650"/>
+    <ext cx="495300" cy="285750"/>
     <pic>
       <nvPicPr>
         <cNvPr id="1" name="Image 1" descr="Picture"/>
@@ -251,7 +266,7 @@
       <row>0</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="247650" cy="247650"/>
+    <ext cx="495300" cy="285750"/>
     <pic>
       <nvPicPr>
         <cNvPr id="1" name="Image 1" descr="Picture"/>
@@ -281,7 +296,7 @@
       <row>0</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="247650" cy="247650"/>
+    <ext cx="495300" cy="285750"/>
     <pic>
       <nvPicPr>
         <cNvPr id="1" name="Image 1" descr="Picture"/>
@@ -311,7 +326,37 @@
       <row>0</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="247650" cy="247650"/>
+    <ext cx="495300" cy="285750"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="1" name="Image 1" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
+</file>
+
+<file path=xl/drawings/drawing6.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>0</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="495300" cy="285750"/>
     <pic>
       <nvPicPr>
         <cNvPr id="1" name="Image 1" descr="Picture"/>
@@ -629,26 +674,196 @@
     </pic>
     <clientData/>
   </oneCellAnchor>
-</wsDr>
-</file>
-
-<file path=xl/drawings/drawing6.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
       <col>0</col>
       <colOff>0</colOff>
-      <row>0</row>
+      <row>14</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="247650" cy="247650"/>
+    <ext cx="285750" cy="285750"/>
     <pic>
       <nvPicPr>
-        <cNvPr id="1" name="Image 1" descr="Picture"/>
+        <cNvPr id="14" name="Image 14" descr="Picture"/>
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId1"/>
+        <a:blip cstate="print" r:embed="rId14"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>15</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="285750" cy="285750"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="15" name="Image 15" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId15"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>16</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="285750" cy="285750"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="16" name="Image 16" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId16"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>17</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="285750" cy="285750"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="17" name="Image 17" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId17"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>18</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="285750" cy="285750"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="18" name="Image 18" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId18"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>19</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="285750" cy="285750"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="19" name="Image 19" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId19"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>20</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="285750" cy="285750"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="20" name="Image 20" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId20"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>21</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="285750" cy="285750"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="21" name="Image 21" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId21"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -671,7 +886,92 @@
       <row>0</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="247650" cy="247650"/>
+    <ext cx="495300" cy="285750"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="1" name="Image 1" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>3</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="9906000" cy="6600825"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="2" name="Image 2" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId2"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
+</file>
+
+<file path=xl/drawings/drawing8.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>0</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="495300" cy="285750"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="1" name="Image 1" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
+</file>
+
+<file path=xl/drawings/drawing9.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>0</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="495300" cy="285750"/>
     <pic>
       <nvPicPr>
         <cNvPr id="1" name="Image 1" descr="Picture"/>
@@ -981,18 +1281,18 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B13"/>
+  <dimension ref="A1:B14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
-    <col width="95" customWidth="1" min="2" max="2"/>
+    <col width="100" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
-    <row r="1" ht="30" customHeight="1">
+    <row r="1" ht="34" customHeight="1">
       <c r="A1" s="1" t="n"/>
       <c r="B1" s="2" t="inlineStr">
         <is>
-          <t>PepsiCo Demand Forecasting — Project Overview</t>
+          <t>PepsiCo Global Demand Forecasting — Project Overview</t>
         </is>
       </c>
     </row>
@@ -1047,96 +1347,108 @@
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>Portfolio in scope</t>
+          <t>Scope</t>
         </is>
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>Beverages (Pepsi, Mtn Dew, Gatorade, Tropicana, Aquafina, 7UP) + Frito-Lay snacks (Lay's, Doritos, Cheetos, Ruffles) + Quaker foods</t>
+          <t>ALL PepsiCo food &amp; beverage brands across geographies. Illustrative markets: UK, Australia, India, Pakistan (4 shown, 20 distinct brands) — extensible to PepsiCo's 200+ markets.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>Data (proxy)</t>
+          <t>Scaling approach</t>
         </is>
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>M5 Forecasting - Accuracy (Walmart, Kaggle) used as a realistic stand-in for PepsiCo's SKU x store x day sales; a real engagement would use PepsiCo shipment / POS / Nielsen data</t>
+          <t>One GLOBAL model with market x brand x category x store embeddings; transfers learning across geos and cold-starts new-market / new-product launches.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t>Forecast target</t>
+          <t>Data (proxy)</t>
         </is>
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>Units sold per SKU x store x day, 28-day horizon, with uncertainty intervals</t>
+          <t>M5 Forecasting - Accuracy (Walmart, Kaggle) as a realistic stand-in for PepsiCo's SKU x store x day sales; a real engagement would use PepsiCo shipment / POS / Nielsen data per market.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>Primary metric</t>
+          <t>Forecast target</t>
         </is>
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>WRMSSE (M5 metric) + MAE / RMSE / pinball loss</t>
+          <t>Units sold per SKU x store x day, 28-day horizon, with uncertainty intervals</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
         <is>
-          <t>Repository</t>
+          <t>Primary metric</t>
         </is>
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>github.com/sudheerchowdary97/cpg-demand-forecasting (public, personal)</t>
+          <t>WRMSSE (M5 metric) + MAE / RMSE / pinball loss</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
         <is>
-          <t>Guardrails</t>
+          <t>Repository</t>
         </is>
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>No Apple ecosystem; heavy training on cloud GPU only; Mac used for light dev</t>
+          <t>github.com/sudheerchowdary97/cpg-demand-forecasting (public, personal)</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
         <is>
-          <t>This workbook</t>
+          <t>Guardrails</t>
         </is>
       </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>Summary of Task 0 (Foundations &amp; Environment) — business + developer views</t>
+          <t>No Apple ecosystem; heavy training on cloud GPU only; Mac used for light dev</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
         <is>
+          <t>This workbook</t>
+        </is>
+      </c>
+      <c r="B13" s="4" t="inlineStr">
+        <is>
+          <t>Summary of Task 0 (Foundations &amp; Environment) — business + developer views</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
           <t>DISCLAIMER</t>
         </is>
       </c>
-      <c r="B13" s="4" t="inlineStr">
-        <is>
-          <t>Independent learning project; NOT affiliated with or endorsed by PepsiCo. Brand icons/colors are stylized, original representations — not official assets. All trademarks belong to their owners.</t>
+      <c r="B14" s="4" t="inlineStr">
+        <is>
+          <t>Independent learning project; NOT affiliated with or endorsed by PepsiCo. Generated brand tiles are stylized originals; logo/infographic are user-supplied. All trademarks belong to their owners.</t>
         </is>
       </c>
     </row>
@@ -1155,19 +1467,19 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C13"/>
+  <dimension ref="A1:C14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="24" customWidth="1" min="1" max="1"/>
-    <col width="64" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="66" customWidth="1" min="2" max="2"/>
     <col width="42" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
-    <row r="1" ht="30" customHeight="1">
+    <row r="1" ht="34" customHeight="1">
       <c r="A1" s="1" t="n"/>
       <c r="B1" s="2" t="inlineStr">
         <is>
-          <t>Business View — PepsiCo Objectives, Pain Points &amp; Solution</t>
+          <t>Business View — Scaling PepsiCo Forecasting Across Geographies</t>
         </is>
       </c>
     </row>
@@ -1196,12 +1508,12 @@
       </c>
       <c r="B3" s="4" t="inlineStr">
         <is>
-          <t>Forecast demand accurately at store level so the right pack is on the right shelf at the right time across Pepsi, Frito-Lay and Quaker.</t>
+          <t>Forecast demand accurately at store level for every food &amp; beverage brand in every market, so the right pack is on the right shelf at the right time.</t>
         </is>
       </c>
       <c r="C3" s="4" t="inlineStr">
         <is>
-          <t>Directly drives net revenue, availability, and working capital.</t>
+          <t>Directly drives net revenue, availability, and working capital worldwide.</t>
         </is>
       </c>
     </row>
@@ -1213,7 +1525,7 @@
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>~$91B annual net revenue, 20+ billion-dollar brands, products sold in 200+ countries/territories.</t>
+          <t>~$91B net revenue, 20+ billion-dollar brands, products in 200+ countries/territories; thousands of SKUs x thousands of stores x many markets.</t>
         </is>
       </c>
       <c r="C4" s="4" t="inlineStr">
@@ -1225,153 +1537,170 @@
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>Pain point 1 — Stockouts</t>
+          <t>Why multi-geo is hard</t>
         </is>
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>Empty shelves lose the sale and push shoppers to competitor brands.</t>
+          <t>Hemisphere-flipped seasons (Australia summer = Dec-Feb), local festivals (Diwali, Ramadan/Eid, Christmas), local brands (Walkers, Smith's, Kurkure, Sting), currencies, prices and weather.</t>
         </is>
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>Lost sales estimated at ~4% of revenue for typical retailers.</t>
+          <t>A single generic model fails; forecasts must be locally aware.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>Pain point 2 — Waste / freshness</t>
+          <t>Local brand portfolios</t>
         </is>
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>Frito-Lay snacks and chilled Tropicana are freshness-critical; overstock becomes stale/expired.</t>
+          <t>Each market carries a tailored mix (e.g., UK: Walkers + Lipton; AU: Smith's + Solo + Sobe; India/Pakistan: Kurkure + Sting).</t>
         </is>
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>Waste and markdowns directly erode margin.</t>
+          <t>The model must handle market-specific catalogs, not one global list.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>Pain point 3 — DSD complexity</t>
+          <t>Pain point — Stockouts</t>
         </is>
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>Direct-Store-Delivery routes must be stocked per store per day without over/under-loading trucks.</t>
+          <t>Empty shelves lose the sale and push shoppers to competitors.</t>
         </is>
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>Route efficiency and service level depend on the forecast.</t>
+          <t>Lost sales estimated at ~4% of revenue for typical retailers.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t>Pain point 4 — Promotions &amp; events</t>
+          <t>Pain point — Waste / freshness</t>
         </is>
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>Promos, price changes, holidays, sports events and heatwaves cause large demand swings.</t>
+          <t>Snacks and chilled juices are freshness-critical; overstock becomes stale/expired.</t>
         </is>
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>Missed spikes = stockouts; over-forecast = waste.</t>
+          <t>Waste and markdowns directly erode margin.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>Pain point 5 — New product launches</t>
+          <t>Pain point — DSD complexity</t>
         </is>
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>Constant limited-time flavors and NPI have little/no history.</t>
+          <t>Direct-Store-Delivery routes must be stocked per store per day across many markets.</t>
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>Cold-start forecasting is hard and high-stakes.</t>
+          <t>Route efficiency and service level depend on the forecast.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
         <is>
-          <t>Proposed solution</t>
+          <t>Pain point — Promotions &amp; events</t>
         </is>
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>Deep-learning time-series models forecasting SKU x store x day demand with uncertainty, feeding replenishment, DSD, production and promo planning.</t>
+          <t>Promos, price changes, holidays, sports events and heatwaves cause large, market-specific swings.</t>
         </is>
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>Captures seasonality, promotions, weather and cross-brand patterns automatically.</t>
+          <t>Missed spikes = stockouts; over-forecast = waste.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
         <is>
-          <t>Business value</t>
+          <t>Pain point — New launches</t>
         </is>
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>Fewer stockouts, less waste, higher service levels, tighter DSD, and data-driven, auditable planning.</t>
+          <t>Constant limited-time flavors, new products, and new-market entries have little/no history.</t>
         </is>
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
-          <t>Improves both top line (sales) and bottom line (margin).</t>
+          <t>Cold-start forecasting is hard and high-stakes.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
         <is>
-          <t>Pathway to impact</t>
+          <t>Proposed solution</t>
         </is>
       </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>Forecasts -&gt; safety stock &amp; replenishment -&gt; DSD route loads -&gt; production plans -&gt; promo planning; served via a live API + planner dashboard.</t>
+          <t>One GLOBAL deep-learning model with market/brand/category embeddings, forecasting SKU x store x day demand with uncertainty, feeding replenishment, DSD, production and promo planning.</t>
         </is>
       </c>
       <c r="C12" s="4" t="inlineStr">
         <is>
-          <t>Turns model output into daily operational decisions.</t>
+          <t>Learns shared patterns across markets while respecting local behavior; scales to new geos.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
         <is>
+          <t>Business value</t>
+        </is>
+      </c>
+      <c r="B13" s="4" t="inlineStr">
+        <is>
+          <t>Fewer stockouts, less waste, higher service levels, faster new-market rollout, and consistent, auditable planning globally.</t>
+        </is>
+      </c>
+      <c r="C13" s="4" t="inlineStr">
+        <is>
+          <t>Improves both top line (sales) and bottom line (margin) at scale.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
           <t>Task 0 in business terms</t>
         </is>
       </c>
-      <c r="B13" s="4" t="inlineStr">
-        <is>
-          <t>Built a trustworthy, reproducible, vendor-neutral foundation before any modeling.</t>
-        </is>
-      </c>
-      <c r="C13" s="4" t="inlineStr">
-        <is>
-          <t>Ensures results are credible and auditable — reduces project risk.</t>
+      <c r="B14" s="4" t="inlineStr">
+        <is>
+          <t>Built a trustworthy, reproducible, vendor-neutral foundation designed to scale across brands and markets.</t>
+        </is>
+      </c>
+      <c r="C14" s="4" t="inlineStr">
+        <is>
+          <t>De-risks the global rollout before any modeling.</t>
         </is>
       </c>
     </row>
@@ -1394,11 +1723,11 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
-    <col width="62" customWidth="1" min="2" max="2"/>
-    <col width="40" customWidth="1" min="3" max="3"/>
+    <col width="64" customWidth="1" min="2" max="2"/>
+    <col width="38" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
-    <row r="1" ht="30" customHeight="1">
+    <row r="1" ht="34" customHeight="1">
       <c r="A1" s="1" t="n"/>
       <c r="B1" s="2" t="inlineStr">
         <is>
@@ -1431,7 +1760,7 @@
       </c>
       <c r="B3" s="4" t="inlineStr">
         <is>
-          <t>Create a reproducible, industry-standard project skeleton before any DL code.</t>
+          <t>Create a reproducible, industry-standard project skeleton that will scale to multi-geo, multi-brand data.</t>
         </is>
       </c>
       <c r="C3" s="4" t="inlineStr">
@@ -1550,7 +1879,7 @@
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>Reusable PepsiCo-styled icon/theme module powering all task workbooks.</t>
+          <t>Reusable module: real PepsiCo logo + generated brand icons + geo/brand data model driving all task workbooks.</t>
         </is>
       </c>
       <c r="C10" s="4" t="inlineStr">
@@ -1562,17 +1891,17 @@
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
         <is>
-          <t>Data / model hygiene</t>
+          <t>Scale-ready data model</t>
         </is>
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>data/ and models/ git-ignored (DVC-tracked later); folders kept via .gitkeep.</t>
+          <t>Brand/geo master data (kind, market coverage) encoded now to seed market x brand x category features later.</t>
         </is>
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
-          <t>.gitignore + DVC intent</t>
+          <t>BRAND_INFO / GEOS</t>
         </is>
       </c>
     </row>
@@ -1601,7 +1930,7 @@
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>README with full Task 0-18 roadmap; MIT license; this branded summary workbook.</t>
+          <t>README roadmap; MIT license; this branded, multi-geo summary workbook.</t>
         </is>
       </c>
       <c r="C13" s="4" t="inlineStr">
@@ -1650,7 +1979,7 @@
     <col width="45" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
-    <row r="1" ht="30" customHeight="1">
+    <row r="1" ht="34" customHeight="1">
       <c r="A1" s="1" t="n"/>
       <c r="B1" s="2" t="inlineStr">
         <is>
@@ -1848,17 +2177,17 @@
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
         <is>
-          <t>Data/model separation</t>
+          <t>Master data modeling</t>
         </is>
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>Keeping large data &amp; artifacts out of git (DVC later).</t>
+          <t>Encoding brand/geo attributes (kind, market coverage) up front.</t>
         </is>
       </c>
       <c r="C13" s="4" t="inlineStr">
         <is>
-          <t>Keeps repo small; data versioned properly.</t>
+          <t>Seeds the embeddings that let one model scale across geos.</t>
         </is>
       </c>
     </row>
@@ -1870,12 +2199,12 @@
       </c>
       <c r="B14" s="4" t="inlineStr">
         <is>
-          <t>Pinned Python + pinned deps + scripted setup.</t>
+          <t>Pinned Python + pinned deps + scripted setup + regenerable assets.</t>
         </is>
       </c>
       <c r="C14" s="4" t="inlineStr">
         <is>
-          <t>Anyone can rebuild the exact environment.</t>
+          <t>Anyone can rebuild the exact environment and docs.</t>
         </is>
       </c>
     </row>
@@ -1894,264 +2223,122 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D14"/>
+  <dimension ref="A1:C7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="8" customWidth="1" min="1" max="1"/>
-    <col width="22" customWidth="1" min="2" max="2"/>
-    <col width="26" customWidth="1" min="3" max="3"/>
-    <col width="60" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="52" customWidth="1" min="2" max="2"/>
+    <col width="52" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
-    <row r="1" ht="30" customHeight="1">
+    <row r="1" ht="34" customHeight="1">
       <c r="A1" s="1" t="n"/>
       <c r="B1" s="2" t="inlineStr">
         <is>
-          <t>PepsiCo Portfolio in Scope — Brands &amp; Forecasting Relevance</t>
+          <t>Global Brand Matrix — Brands by Market (Food + Beverage)</t>
         </is>
       </c>
     </row>
     <row r="2" ht="22" customHeight="1">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>Icon</t>
+          <t>Market</t>
         </is>
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>Brand</t>
+          <t>Food Brands (5)</t>
         </is>
       </c>
       <c r="C2" s="3" t="inlineStr">
         <is>
-          <t>Category</t>
-        </is>
-      </c>
-      <c r="D2" s="3" t="inlineStr">
-        <is>
-          <t>Forecasting relevance</t>
+          <t>Beverage Brands (5)</t>
         </is>
       </c>
     </row>
     <row r="3" ht="34" customHeight="1">
-      <c r="A3" s="4" t="inlineStr"/>
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>🇬🇧 UK
+Great tasting brands for British lifestyles.</t>
+        </is>
+      </c>
       <c r="B3" s="4" t="inlineStr">
         <is>
-          <t>🥤 Pepsi</t>
+          <t>Walkers, Doritos, Quaker, Cheetos, Ruffles</t>
         </is>
       </c>
       <c r="C3" s="4" t="inlineStr">
         <is>
-          <t>Carbonated soft drinks</t>
-        </is>
-      </c>
-      <c r="D3" s="4" t="inlineStr">
-        <is>
-          <t>Top-volume CSD; strong summer &amp; holiday peaks, heavy promo lift.</t>
+          <t>Pepsi, Pepsi Max, 7UP, Tropicana, Lipton</t>
         </is>
       </c>
     </row>
     <row r="4" ht="34" customHeight="1">
-      <c r="A4" s="4" t="inlineStr"/>
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>🇦🇺 Australia
+Iconic brands for an active, outdoor lifestyle.</t>
+        </is>
+      </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>🏔 Mountain Dew</t>
+          <t>Smith's, Doritos, Red Rock Deli, Cheetos, Quaker</t>
         </is>
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>Carbonated soft drinks</t>
-        </is>
-      </c>
-      <c r="D4" s="4" t="inlineStr">
-        <is>
-          <t>Youth-skewed CSD; limited-time flavors drive sharp launch spikes.</t>
+          <t>Pepsi, Solo, Mountain Dew, Gatorade, Sobe</t>
         </is>
       </c>
     </row>
     <row r="5" ht="34" customHeight="1">
-      <c r="A5" s="4" t="inlineStr"/>
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>🇮🇳 India
+Popular brands for every occasion.</t>
+        </is>
+      </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>⚡ Gatorade</t>
+          <t>Lay's, Kurkure, Doritos, Quaker, Cheetos</t>
         </is>
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>Sports drinks</t>
-        </is>
-      </c>
-      <c r="D5" s="4" t="inlineStr">
-        <is>
-          <t>Sports/heat-driven; demand tracks temperature and sports seasons.</t>
+          <t>Pepsi, Mountain Dew, 7UP, Tropicana, Sting</t>
         </is>
       </c>
     </row>
     <row r="6" ht="34" customHeight="1">
-      <c r="A6" s="4" t="inlineStr"/>
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>🇵🇰 Pakistan
+Great taste, every day.</t>
+        </is>
+      </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>🍊 Tropicana</t>
+          <t>Lay's, Kurkure, Doritos, Quaker, Cheetos</t>
         </is>
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>Chilled juices</t>
-        </is>
-      </c>
-      <c r="D6" s="4" t="inlineStr">
-        <is>
-          <t>Chilled juice; short shelf life, breakfast + winter-cold seasonality.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="34" customHeight="1">
-      <c r="A7" s="4" t="inlineStr"/>
-      <c r="B7" s="4" t="inlineStr">
-        <is>
-          <t>💧 Aquafina</t>
-        </is>
-      </c>
-      <c r="C7" s="4" t="inlineStr">
-        <is>
-          <t>Bottled water</t>
-        </is>
-      </c>
-      <c r="D7" s="4" t="inlineStr">
-        <is>
-          <t>Water; strong summer and heatwave sensitivity.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="34" customHeight="1">
-      <c r="A8" s="4" t="inlineStr"/>
-      <c r="B8" s="4" t="inlineStr">
-        <is>
-          <t>🥤 7UP</t>
-        </is>
-      </c>
-      <c r="C8" s="4" t="inlineStr">
-        <is>
-          <t>Carbonated soft drinks</t>
-        </is>
-      </c>
-      <c r="D8" s="4" t="inlineStr">
-        <is>
-          <t>CSD; festive/holiday and mixer demand.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="34" customHeight="1">
-      <c r="A9" s="4" t="inlineStr"/>
-      <c r="B9" s="4" t="inlineStr">
-        <is>
-          <t>🥔 Lay's</t>
-        </is>
-      </c>
-      <c r="C9" s="4" t="inlineStr">
-        <is>
-          <t>Salty snacks (Frito-Lay)</t>
-        </is>
-      </c>
-      <c r="D9" s="4" t="inlineStr">
-        <is>
-          <t>DSD salty snack; freshness-critical, very high promo frequency.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="34" customHeight="1">
-      <c r="A10" s="4" t="inlineStr"/>
-      <c r="B10" s="4" t="inlineStr">
-        <is>
-          <t>🔺 Doritos</t>
-        </is>
-      </c>
-      <c r="C10" s="4" t="inlineStr">
-        <is>
-          <t>Salty snacks (Frito-Lay)</t>
-        </is>
-      </c>
-      <c r="D10" s="4" t="inlineStr">
-        <is>
-          <t>Snack; big-game/event and limited-edition spikes.</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="34" customHeight="1">
-      <c r="A11" s="4" t="inlineStr"/>
-      <c r="B11" s="4" t="inlineStr">
-        <is>
-          <t>🐆 Cheetos</t>
-        </is>
-      </c>
-      <c r="C11" s="4" t="inlineStr">
-        <is>
-          <t>Salty snacks (Frito-Lay)</t>
-        </is>
-      </c>
-      <c r="D11" s="4" t="inlineStr">
-        <is>
-          <t>Snack; steady base with promo-driven lift.</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="34" customHeight="1">
-      <c r="A12" s="4" t="inlineStr"/>
-      <c r="B12" s="4" t="inlineStr">
-        <is>
-          <t>🥔 Ruffles</t>
-        </is>
-      </c>
-      <c r="C12" s="4" t="inlineStr">
-        <is>
-          <t>Salty snacks (Frito-Lay)</t>
-        </is>
-      </c>
-      <c r="D12" s="4" t="inlineStr">
-        <is>
-          <t>Snack; party/occasion and promo sensitive.</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="34" customHeight="1">
-      <c r="A13" s="4" t="inlineStr"/>
-      <c r="B13" s="4" t="inlineStr">
-        <is>
-          <t>🥣 Quaker</t>
-        </is>
-      </c>
-      <c r="C13" s="4" t="inlineStr">
-        <is>
-          <t>Foods / oats</t>
-        </is>
-      </c>
-      <c r="D13" s="4" t="inlineStr">
-        <is>
-          <t>Ambient breakfast; longer shelf life, winter skew.</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="34" customHeight="1">
-      <c r="A14" s="4" t="inlineStr"/>
-      <c r="B14" s="4" t="inlineStr">
-        <is>
-          <t>⚡ Rockstar</t>
-        </is>
-      </c>
-      <c r="C14" s="4" t="inlineStr">
-        <is>
-          <t>Energy drinks</t>
-        </is>
-      </c>
-      <c r="D14" s="4" t="inlineStr">
-        <is>
-          <t>Energy; convenience-channel, weekday skew.</t>
+          <t>Pepsi, 7UP, Mountain Dew, Aquafina, Sting</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="30" customHeight="1">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>Illustrative 4 of PepsiCo's 200+ markets. One global model scales to new markets via market/brand/category embeddings + hierarchical forecasting.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="B1:D1"/>
+  <mergeCells count="2">
+    <mergeCell ref="B1:C1"/>
+    <mergeCell ref="A7:C7"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -2164,561 +2351,508 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E21"/>
+  <dimension ref="A1:E22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="7" customWidth="1" min="1" max="1"/>
-    <col width="38" customWidth="1" min="2" max="2"/>
-    <col width="32" customWidth="1" min="3" max="3"/>
-    <col width="34" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="24" customWidth="1" min="4" max="4"/>
+    <col width="34" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
-    <row r="1" ht="30" customHeight="1">
+    <row r="1" ht="34" customHeight="1">
       <c r="A1" s="1" t="n"/>
       <c r="B1" s="2" t="inlineStr">
         <is>
-          <t>Full Roadmap — Task 0 to 18</t>
+          <t>Brand Portfolio in Scope — 20 Brands Across Markets</t>
         </is>
       </c>
     </row>
     <row r="2" ht="22" customHeight="1">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>Task</t>
+          <t>Icon</t>
         </is>
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>Name</t>
+          <t>Brand</t>
         </is>
       </c>
       <c r="C2" s="3" t="inlineStr">
         <is>
-          <t>Core DL concept</t>
+          <t>Type</t>
         </is>
       </c>
       <c r="D2" s="3" t="inlineStr">
         <is>
-          <t>Engineering skill</t>
+          <t>Category</t>
         </is>
       </c>
       <c r="E2" s="3" t="inlineStr">
         <is>
-          <t>Status</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="5" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="B3" s="5" t="inlineStr">
-        <is>
-          <t>Foundations &amp; environment</t>
-        </is>
-      </c>
-      <c r="C3" s="5" t="inlineStr">
-        <is>
-          <t>— (tooling)</t>
-        </is>
-      </c>
-      <c r="D3" s="5" t="inlineStr">
-        <is>
-          <t>repo layout, venv, linting, tests</t>
-        </is>
-      </c>
-      <c r="E3" s="5" t="inlineStr">
-        <is>
-          <t>Done ✅</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="4" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>Markets in scope</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="34" customHeight="1">
+      <c r="A3" s="4" t="inlineStr"/>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>🥔 Lay's</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>Food</t>
+        </is>
+      </c>
+      <c r="D3" s="4" t="inlineStr">
+        <is>
+          <t>Salty snacks (Frito-Lay)</t>
+        </is>
+      </c>
+      <c r="E3" s="4" t="inlineStr">
+        <is>
+          <t>India, Pakistan</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="34" customHeight="1">
+      <c r="A4" s="4" t="inlineStr"/>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>Problem framing &amp; data (DVC)</t>
+          <t>🥔 Walkers</t>
         </is>
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>forecast task formulation</t>
+          <t>Food</t>
         </is>
       </c>
       <c r="D4" s="4" t="inlineStr">
         <is>
-          <t>data versioning</t>
+          <t>Salty snacks (Frito-Lay)</t>
         </is>
       </c>
       <c r="E4" s="4" t="inlineStr">
         <is>
-          <t>Next</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="4" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
+          <t>UK</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="34" customHeight="1">
+      <c r="A5" s="4" t="inlineStr"/>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>EDA &amp; time-series understanding</t>
+          <t>🥔 Smith's</t>
         </is>
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>seasonality, stationarity</t>
+          <t>Food</t>
         </is>
       </c>
       <c r="D5" s="4" t="inlineStr">
         <is>
-          <t>reproducible notebooks</t>
+          <t>Salty snacks (Frito-Lay)</t>
         </is>
       </c>
       <c r="E5" s="4" t="inlineStr">
         <is>
-          <t>Planned</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="4" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
+          <t>Australia</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="34" customHeight="1">
+      <c r="A6" s="4" t="inlineStr"/>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>Data pipeline &amp; feature engineering</t>
+          <t>🔺 Doritos</t>
         </is>
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>windowing, embeddings</t>
+          <t>Food</t>
         </is>
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>leakage-free ETL as code</t>
+          <t>Salty snacks (Frito-Lay)</t>
         </is>
       </c>
       <c r="E6" s="4" t="inlineStr">
         <is>
-          <t>Planned</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="4" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
+          <t>UK, Australia, India, Pakistan</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="34" customHeight="1">
+      <c r="A7" s="4" t="inlineStr"/>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>Classical baselines &amp; eval harness</t>
+          <t>🐆 Cheetos</t>
         </is>
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>why baselines matter</t>
+          <t>Food</t>
         </is>
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t>WRMSSE, backtesting, tracking</t>
+          <t>Salty snacks (Frito-Lay)</t>
         </is>
       </c>
       <c r="E7" s="4" t="inlineStr">
         <is>
-          <t>Planned</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="4" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
-      </c>
+          <t>UK, Australia, India, Pakistan</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="34" customHeight="1">
+      <c r="A8" s="4" t="inlineStr"/>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>MLP forecaster</t>
+          <t>🥔 Ruffles</t>
         </is>
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>MLPs, backprop, regularization</t>
+          <t>Food</t>
         </is>
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>Lightning training loop</t>
+          <t>Salty snacks (Frito-Lay)</t>
         </is>
       </c>
       <c r="E8" s="4" t="inlineStr">
         <is>
-          <t>Planned</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="4" t="inlineStr">
-        <is>
-          <t>6</t>
-        </is>
-      </c>
+          <t>UK</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="34" customHeight="1">
+      <c r="A9" s="4" t="inlineStr"/>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>RNN -&gt; LSTM -&gt; GRU</t>
+          <t>🥣 Quaker</t>
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>recurrence, gating</t>
+          <t>Food</t>
         </is>
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>GPU training discipline</t>
+          <t>Foods / oats</t>
         </is>
       </c>
       <c r="E9" s="4" t="inlineStr">
         <is>
-          <t>Planned</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="4" t="inlineStr">
-        <is>
-          <t>7</t>
-        </is>
-      </c>
+          <t>UK, Australia, India, Pakistan</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="34" customHeight="1">
+      <c r="A10" s="4" t="inlineStr"/>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>Seq2Seq + Attention</t>
+          <t>🌶 Kurkure</t>
         </is>
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>attention, multi-horizon</t>
+          <t>Food</t>
         </is>
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>attention visualization</t>
+          <t>Salty snacks (local)</t>
         </is>
       </c>
       <c r="E10" s="4" t="inlineStr">
         <is>
-          <t>Planned</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="4" t="inlineStr">
-        <is>
-          <t>8</t>
-        </is>
-      </c>
+          <t>India, Pakistan</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="34" customHeight="1">
+      <c r="A11" s="4" t="inlineStr"/>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>Temporal Conv Nets (TCN)</t>
+          <t>🥔 Red Rock Deli</t>
         </is>
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
-          <t>dilated causal convolution</t>
+          <t>Food</t>
         </is>
       </c>
       <c r="D11" s="4" t="inlineStr">
         <is>
-          <t>architecture ablation</t>
+          <t>Premium salty snacks</t>
         </is>
       </c>
       <c r="E11" s="4" t="inlineStr">
         <is>
-          <t>Planned</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="4" t="inlineStr">
-        <is>
-          <t>9</t>
-        </is>
-      </c>
+          <t>Australia</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="34" customHeight="1">
+      <c r="A12" s="4" t="inlineStr"/>
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>Transformer / TFT</t>
+          <t>🥤 Pepsi</t>
         </is>
       </c>
       <c r="C12" s="4" t="inlineStr">
         <is>
-          <t>self-attention, interpretability</t>
+          <t>Beverage</t>
         </is>
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
-          <t>large-model training</t>
+          <t>Carbonated soft drinks</t>
         </is>
       </c>
       <c r="E12" s="4" t="inlineStr">
         <is>
-          <t>Planned</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="4" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
-      </c>
+          <t>UK, Australia, India, Pakistan</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="34" customHeight="1">
+      <c r="A13" s="4" t="inlineStr"/>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>Probabilistic (DeepAR / N-BEATS)</t>
+          <t>🥤 Pepsi Max</t>
         </is>
       </c>
       <c r="C13" s="4" t="inlineStr">
         <is>
-          <t>uncertainty, intermittency</t>
+          <t>Beverage</t>
         </is>
       </c>
       <c r="D13" s="4" t="inlineStr">
         <is>
-          <t>calibration</t>
+          <t>Carbonated soft drinks</t>
         </is>
       </c>
       <c r="E13" s="4" t="inlineStr">
         <is>
-          <t>Planned</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="4" t="inlineStr">
-        <is>
-          <t>11</t>
-        </is>
-      </c>
+          <t>UK</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="34" customHeight="1">
+      <c r="A14" s="4" t="inlineStr"/>
       <c r="B14" s="4" t="inlineStr">
         <is>
-          <t>Tracking, HPO &amp; model selection</t>
+          <t>🥤 7UP</t>
         </is>
       </c>
       <c r="C14" s="4" t="inlineStr">
         <is>
-          <t>HPO, bias/variance</t>
+          <t>Beverage</t>
         </is>
       </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
-          <t>Optuna + MLflow</t>
+          <t>Carbonated soft drinks</t>
         </is>
       </c>
       <c r="E14" s="4" t="inlineStr">
         <is>
-          <t>Planned</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="4" t="inlineStr">
-        <is>
-          <t>12</t>
-        </is>
-      </c>
+          <t>UK, India, Pakistan</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="34" customHeight="1">
+      <c r="A15" s="4" t="inlineStr"/>
       <c r="B15" s="4" t="inlineStr">
         <is>
-          <t>Cloud full-scale training</t>
+          <t>🍊 Tropicana</t>
         </is>
       </c>
       <c r="C15" s="4" t="inlineStr">
         <is>
-          <t>mixed precision, checkpointing</t>
+          <t>Beverage</t>
         </is>
       </c>
       <c r="D15" s="4" t="inlineStr">
         <is>
-          <t>training-as-code</t>
+          <t>Juices</t>
         </is>
       </c>
       <c r="E15" s="4" t="inlineStr">
         <is>
-          <t>Planned</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="4" t="inlineStr">
-        <is>
-          <t>13</t>
-        </is>
-      </c>
+          <t>UK, India</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="34" customHeight="1">
+      <c r="A16" s="4" t="inlineStr"/>
       <c r="B16" s="4" t="inlineStr">
         <is>
-          <t>Export &amp; optimize (ONNX / quantize)</t>
+          <t>🍵 Lipton</t>
         </is>
       </c>
       <c r="C16" s="4" t="inlineStr">
         <is>
-          <t>graph export, quantization</t>
+          <t>Beverage</t>
         </is>
       </c>
       <c r="D16" s="4" t="inlineStr">
         <is>
-          <t>perf benchmarking</t>
+          <t>Ready-to-drink tea</t>
         </is>
       </c>
       <c r="E16" s="4" t="inlineStr">
         <is>
-          <t>Planned</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="4" t="inlineStr">
-        <is>
-          <t>14</t>
-        </is>
-      </c>
+          <t>UK</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="34" customHeight="1">
+      <c r="A17" s="4" t="inlineStr"/>
       <c r="B17" s="4" t="inlineStr">
         <is>
-          <t>Serving API (FastAPI + Docker)</t>
+          <t>🍋 Solo</t>
         </is>
       </c>
       <c r="C17" s="4" t="inlineStr">
         <is>
-          <t>inference-time preprocessing</t>
+          <t>Beverage</t>
         </is>
       </c>
       <c r="D17" s="4" t="inlineStr">
         <is>
-          <t>API design, containers</t>
+          <t>Carbonated soft drinks</t>
         </is>
       </c>
       <c r="E17" s="4" t="inlineStr">
         <is>
-          <t>Planned</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="4" t="inlineStr">
-        <is>
-          <t>15</t>
-        </is>
-      </c>
+          <t>Australia</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="34" customHeight="1">
+      <c r="A18" s="4" t="inlineStr"/>
       <c r="B18" s="4" t="inlineStr">
         <is>
-          <t>Cloud deploy + CI/CD</t>
+          <t>🏔 Mountain Dew</t>
         </is>
       </c>
       <c r="C18" s="4" t="inlineStr">
         <is>
-          <t>production readiness</t>
+          <t>Beverage</t>
         </is>
       </c>
       <c r="D18" s="4" t="inlineStr">
         <is>
-          <t>Cloud Run/Render, GitHub Actions</t>
+          <t>Carbonated soft drinks</t>
         </is>
       </c>
       <c r="E18" s="4" t="inlineStr">
         <is>
-          <t>Planned</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="4" t="inlineStr">
-        <is>
-          <t>16</t>
-        </is>
-      </c>
+          <t>Australia, India, Pakistan</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="34" customHeight="1">
+      <c r="A19" s="4" t="inlineStr"/>
       <c r="B19" s="4" t="inlineStr">
         <is>
-          <t>Monitoring, drift &amp; retraining</t>
+          <t>⚡ Gatorade</t>
         </is>
       </c>
       <c r="C19" s="4" t="inlineStr">
         <is>
-          <t>distribution shift</t>
+          <t>Beverage</t>
         </is>
       </c>
       <c r="D19" s="4" t="inlineStr">
         <is>
-          <t>observability</t>
+          <t>Sports drinks</t>
         </is>
       </c>
       <c r="E19" s="4" t="inlineStr">
         <is>
-          <t>Planned</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="4" t="inlineStr">
-        <is>
-          <t>17</t>
-        </is>
-      </c>
+          <t>Australia</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="34" customHeight="1">
+      <c r="A20" s="4" t="inlineStr"/>
       <c r="B20" s="4" t="inlineStr">
         <is>
-          <t>Demo app + LLM insight layer</t>
+          <t>🦎 Sobe</t>
         </is>
       </c>
       <c r="C20" s="4" t="inlineStr">
         <is>
-          <t>communicating uncertainty</t>
+          <t>Beverage</t>
         </is>
       </c>
       <c r="D20" s="4" t="inlineStr">
         <is>
-          <t>Streamlit, prompt design</t>
+          <t>Enhanced / flavored drinks</t>
         </is>
       </c>
       <c r="E20" s="4" t="inlineStr">
         <is>
-          <t>Planned</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="4" t="inlineStr">
-        <is>
-          <t>18</t>
-        </is>
-      </c>
+          <t>Australia</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="34" customHeight="1">
+      <c r="A21" s="4" t="inlineStr"/>
       <c r="B21" s="4" t="inlineStr">
         <is>
-          <t>Docs, presentation &amp; portfolio</t>
+          <t>⚡ Sting</t>
         </is>
       </c>
       <c r="C21" s="4" t="inlineStr">
         <is>
-          <t>synthesis</t>
+          <t>Beverage</t>
         </is>
       </c>
       <c r="D21" s="4" t="inlineStr">
         <is>
-          <t>technical writing, Keynote-HTML</t>
+          <t>Energy drinks</t>
         </is>
       </c>
       <c r="E21" s="4" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>India, Pakistan</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="34" customHeight="1">
+      <c r="A22" s="4" t="inlineStr"/>
+      <c r="B22" s="4" t="inlineStr">
+        <is>
+          <t>💧 Aquafina</t>
+        </is>
+      </c>
+      <c r="C22" s="4" t="inlineStr">
+        <is>
+          <t>Beverage</t>
+        </is>
+      </c>
+      <c r="D22" s="4" t="inlineStr">
+        <is>
+          <t>Bottled water</t>
+        </is>
+      </c>
+      <c r="E22" s="4" t="inlineStr">
+        <is>
+          <t>Pakistan</t>
         </is>
       </c>
     </row>
@@ -2737,14 +2871,623 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B14"/>
+  <dimension ref="A1:B2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="20" customWidth="1" min="1" max="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="34" customHeight="1">
+      <c r="A1" s="1" t="n"/>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>Loved Brands. Local Markets. — Global Portfolio Map</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="6" t="inlineStr">
+        <is>
+          <t>Source: user-supplied PepsiCo portfolio infographic (docs/brands_icons/Brands_Geos.png).</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="B1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E21"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="7" customWidth="1" min="1" max="1"/>
+    <col width="38" customWidth="1" min="2" max="2"/>
+    <col width="36" customWidth="1" min="3" max="3"/>
+    <col width="32" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="34" customHeight="1">
+      <c r="A1" s="1" t="n"/>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>Full Roadmap — Task 0 to 18 (multi-geo, multi-brand)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="22" customHeight="1">
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t>Task</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="C2" s="3" t="inlineStr">
+        <is>
+          <t>Core DL concept</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="inlineStr">
+        <is>
+          <t>Engineering skill</t>
+        </is>
+      </c>
+      <c r="E2" s="3" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="7" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="B3" s="7" t="inlineStr">
+        <is>
+          <t>Foundations &amp; environment</t>
+        </is>
+      </c>
+      <c r="C3" s="7" t="inlineStr">
+        <is>
+          <t>— (tooling)</t>
+        </is>
+      </c>
+      <c r="D3" s="7" t="inlineStr">
+        <is>
+          <t>repo layout, venv, linting, tests</t>
+        </is>
+      </c>
+      <c r="E3" s="7" t="inlineStr">
+        <is>
+          <t>Done ✅</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>Problem framing &amp; data (DVC)</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>forecast task formulation</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="inlineStr">
+        <is>
+          <t>data versioning</t>
+        </is>
+      </c>
+      <c r="E4" s="4" t="inlineStr">
+        <is>
+          <t>Next</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>EDA &amp; time-series understanding</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>seasonality, stationarity</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>reproducible notebooks</t>
+        </is>
+      </c>
+      <c r="E5" s="4" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>Data pipeline &amp; feature engineering</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>windowing, market/brand embeddings</t>
+        </is>
+      </c>
+      <c r="D6" s="4" t="inlineStr">
+        <is>
+          <t>leakage-free ETL as code</t>
+        </is>
+      </c>
+      <c r="E6" s="4" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>Classical baselines &amp; eval harness</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>why baselines matter</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t>WRMSSE, backtesting, tracking</t>
+        </is>
+      </c>
+      <c r="E7" s="4" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>MLP forecaster</t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="inlineStr">
+        <is>
+          <t>MLPs, backprop, regularization</t>
+        </is>
+      </c>
+      <c r="D8" s="4" t="inlineStr">
+        <is>
+          <t>Lightning training loop</t>
+        </is>
+      </c>
+      <c r="E8" s="4" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>RNN -&gt; LSTM -&gt; GRU</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="inlineStr">
+        <is>
+          <t>recurrence, gating</t>
+        </is>
+      </c>
+      <c r="D9" s="4" t="inlineStr">
+        <is>
+          <t>GPU training discipline</t>
+        </is>
+      </c>
+      <c r="E9" s="4" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="B10" s="4" t="inlineStr">
+        <is>
+          <t>Seq2Seq + Attention</t>
+        </is>
+      </c>
+      <c r="C10" s="4" t="inlineStr">
+        <is>
+          <t>attention, multi-horizon</t>
+        </is>
+      </c>
+      <c r="D10" s="4" t="inlineStr">
+        <is>
+          <t>attention visualization</t>
+        </is>
+      </c>
+      <c r="E10" s="4" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="B11" s="4" t="inlineStr">
+        <is>
+          <t>Temporal Conv Nets (TCN)</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="inlineStr">
+        <is>
+          <t>dilated causal convolution</t>
+        </is>
+      </c>
+      <c r="D11" s="4" t="inlineStr">
+        <is>
+          <t>architecture ablation</t>
+        </is>
+      </c>
+      <c r="E11" s="4" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B12" s="4" t="inlineStr">
+        <is>
+          <t>Transformer / TFT</t>
+        </is>
+      </c>
+      <c r="C12" s="4" t="inlineStr">
+        <is>
+          <t>self-attention, static covariates (geo/brand)</t>
+        </is>
+      </c>
+      <c r="D12" s="4" t="inlineStr">
+        <is>
+          <t>large-model training</t>
+        </is>
+      </c>
+      <c r="E12" s="4" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="B13" s="4" t="inlineStr">
+        <is>
+          <t>Probabilistic (DeepAR / N-BEATS)</t>
+        </is>
+      </c>
+      <c r="C13" s="4" t="inlineStr">
+        <is>
+          <t>uncertainty, intermittency</t>
+        </is>
+      </c>
+      <c r="D13" s="4" t="inlineStr">
+        <is>
+          <t>calibration</t>
+        </is>
+      </c>
+      <c r="E13" s="4" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="B14" s="4" t="inlineStr">
+        <is>
+          <t>Tracking, HPO &amp; model selection</t>
+        </is>
+      </c>
+      <c r="C14" s="4" t="inlineStr">
+        <is>
+          <t>HPO, bias/variance</t>
+        </is>
+      </c>
+      <c r="D14" s="4" t="inlineStr">
+        <is>
+          <t>Optuna + MLflow</t>
+        </is>
+      </c>
+      <c r="E14" s="4" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="B15" s="4" t="inlineStr">
+        <is>
+          <t>Cloud full-scale training</t>
+        </is>
+      </c>
+      <c r="C15" s="4" t="inlineStr">
+        <is>
+          <t>global model across all markets</t>
+        </is>
+      </c>
+      <c r="D15" s="4" t="inlineStr">
+        <is>
+          <t>training-as-code</t>
+        </is>
+      </c>
+      <c r="E15" s="4" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
+      <c r="B16" s="4" t="inlineStr">
+        <is>
+          <t>Export &amp; optimize (ONNX / quantize)</t>
+        </is>
+      </c>
+      <c r="C16" s="4" t="inlineStr">
+        <is>
+          <t>graph export, quantization</t>
+        </is>
+      </c>
+      <c r="D16" s="4" t="inlineStr">
+        <is>
+          <t>perf benchmarking</t>
+        </is>
+      </c>
+      <c r="E16" s="4" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+      <c r="B17" s="4" t="inlineStr">
+        <is>
+          <t>Serving API (FastAPI + Docker)</t>
+        </is>
+      </c>
+      <c r="C17" s="4" t="inlineStr">
+        <is>
+          <t>inference-time preprocessing</t>
+        </is>
+      </c>
+      <c r="D17" s="4" t="inlineStr">
+        <is>
+          <t>API design, containers</t>
+        </is>
+      </c>
+      <c r="E17" s="4" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="B18" s="4" t="inlineStr">
+        <is>
+          <t>Cloud deploy + CI/CD</t>
+        </is>
+      </c>
+      <c r="C18" s="4" t="inlineStr">
+        <is>
+          <t>production readiness</t>
+        </is>
+      </c>
+      <c r="D18" s="4" t="inlineStr">
+        <is>
+          <t>Cloud Run/Render, GitHub Actions</t>
+        </is>
+      </c>
+      <c r="E18" s="4" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="B19" s="4" t="inlineStr">
+        <is>
+          <t>Monitoring, drift &amp; retraining</t>
+        </is>
+      </c>
+      <c r="C19" s="4" t="inlineStr">
+        <is>
+          <t>distribution shift per market</t>
+        </is>
+      </c>
+      <c r="D19" s="4" t="inlineStr">
+        <is>
+          <t>observability</t>
+        </is>
+      </c>
+      <c r="E19" s="4" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>17</t>
+        </is>
+      </c>
+      <c r="B20" s="4" t="inlineStr">
+        <is>
+          <t>Demo app + LLM insight layer</t>
+        </is>
+      </c>
+      <c r="C20" s="4" t="inlineStr">
+        <is>
+          <t>communicating uncertainty</t>
+        </is>
+      </c>
+      <c r="D20" s="4" t="inlineStr">
+        <is>
+          <t>Streamlit, prompt design</t>
+        </is>
+      </c>
+      <c r="E20" s="4" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
+      <c r="B21" s="4" t="inlineStr">
+        <is>
+          <t>Docs, presentation &amp; portfolio</t>
+        </is>
+      </c>
+      <c r="C21" s="4" t="inlineStr">
+        <is>
+          <t>synthesis</t>
+        </is>
+      </c>
+      <c r="D21" s="4" t="inlineStr">
+        <is>
+          <t>technical writing, Keynote-HTML</t>
+        </is>
+      </c>
+      <c r="E21" s="4" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="B1:E1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="65" customWidth="1" min="1" max="1"/>
     <col width="14" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
-    <row r="1" ht="30" customHeight="1">
+    <row r="1" ht="34" customHeight="1">
       <c r="A1" s="1" t="n"/>
       <c r="B1" s="2" t="inlineStr">
         <is>
@@ -2765,144 +3508,156 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="5" t="inlineStr">
+      <c r="A3" s="7" t="inlineStr">
         <is>
           <t>src/ layout package (cpg_forecast) installed editable</t>
         </is>
       </c>
-      <c r="B3" s="5" t="inlineStr">
+      <c r="B3" s="7" t="inlineStr">
         <is>
           <t>Done ✅</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="5" t="inlineStr">
+      <c r="A4" s="7" t="inlineStr">
         <is>
           <t>Python 3.12 virtual environment</t>
         </is>
       </c>
-      <c r="B4" s="5" t="inlineStr">
+      <c r="B4" s="7" t="inlineStr">
         <is>
           <t>Done ✅</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="5" t="inlineStr">
+      <c r="A5" s="7" t="inlineStr">
         <is>
           <t>pyproject.toml with dev + docs extras</t>
         </is>
       </c>
-      <c r="B5" s="5" t="inlineStr">
+      <c r="B5" s="7" t="inlineStr">
         <is>
           <t>Done ✅</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="5" t="inlineStr">
+      <c r="A6" s="7" t="inlineStr">
         <is>
           <t>ruff + black wired via pre-commit</t>
         </is>
       </c>
-      <c r="B6" s="5" t="inlineStr">
+      <c r="B6" s="7" t="inlineStr">
         <is>
           <t>Done ✅</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="5" t="inlineStr">
+      <c r="A7" s="7" t="inlineStr">
         <is>
           <t>Passing smoke tests (pytest)</t>
         </is>
       </c>
-      <c r="B7" s="5" t="inlineStr">
+      <c r="B7" s="7" t="inlineStr">
         <is>
           <t>Done ✅</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="5" t="inlineStr">
+      <c r="A8" s="7" t="inlineStr">
         <is>
           <t>Makefile (setup/lint/format/test/summary)</t>
         </is>
       </c>
-      <c r="B8" s="5" t="inlineStr">
+      <c r="B8" s="7" t="inlineStr">
         <is>
           <t>Done ✅</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="5" t="inlineStr">
+      <c r="A9" s="7" t="inlineStr">
         <is>
           <t>.gitignore + DVC-ready data/model folders</t>
         </is>
       </c>
-      <c r="B9" s="5" t="inlineStr">
+      <c r="B9" s="7" t="inlineStr">
         <is>
           <t>Done ✅</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="5" t="inlineStr">
+      <c r="A10" s="7" t="inlineStr">
         <is>
           <t>README with full roadmap + MIT LICENSE</t>
         </is>
       </c>
-      <c r="B10" s="5" t="inlineStr">
+      <c r="B10" s="7" t="inlineStr">
         <is>
           <t>Done ✅</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="5" t="inlineStr">
+      <c r="A11" s="7" t="inlineStr">
         <is>
           <t>Personal (non-Apple) git identity</t>
         </is>
       </c>
-      <c r="B11" s="5" t="inlineStr">
+      <c r="B11" s="7" t="inlineStr">
         <is>
           <t>Done ✅</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="5" t="inlineStr">
+      <c r="A12" s="7" t="inlineStr">
         <is>
           <t>Repo created &amp; pushed to personal GitHub</t>
         </is>
       </c>
-      <c r="B12" s="5" t="inlineStr">
+      <c r="B12" s="7" t="inlineStr">
         <is>
           <t>Done ✅</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="5" t="inlineStr">
-        <is>
-          <t>PepsiCo-styled branding module (icons/theme)</t>
-        </is>
-      </c>
-      <c r="B13" s="5" t="inlineStr">
+      <c r="A13" s="7" t="inlineStr">
+        <is>
+          <t>PepsiCo branding: real logo + generated brand icons</t>
+        </is>
+      </c>
+      <c r="B13" s="7" t="inlineStr">
         <is>
           <t>Done ✅</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="5" t="inlineStr">
+      <c r="A14" s="7" t="inlineStr">
+        <is>
+          <t>Multi-geo, multi-brand scope defined (matrix + portfolio)</t>
+        </is>
+      </c>
+      <c r="B14" s="7" t="inlineStr">
+        <is>
+          <t>Done ✅</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="7" t="inlineStr">
         <is>
           <t>Business + developer summary workbook (this file)</t>
         </is>
       </c>
-      <c r="B14" s="5" t="inlineStr">
+      <c r="B15" s="7" t="inlineStr">
         <is>
           <t>Done ✅</t>
         </is>

</xml_diff>

<commit_message>
Task 0 docs: reframe architecture to evidence-driven Local->Global->Hybrid
- drop 'one global model is final' framing in Overview + Business
- new 'Architecture' sheet: local baselines / global multi-series w/ embeddings /
  segmented globals (Beverages vs Snacks) / geo fine-tuning / hierarchical
  reconciliation / selection-by-backtesting + data-residency (learning vs prod)
- roadmap Tasks 4/9/12: local baseline -> global model -> market comparison ->
  hybrid refinement; global NOT assumed to beat local
- README: matching roadmap rows + Architecture & data-residency section
</commit_message>
<xml_diff>
--- a/docs/Task0_Summary.xlsx
+++ b/docs/Task0_Summary.xlsx
@@ -14,8 +14,9 @@
     <sheet name="Global Brand Matrix" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="Brand Portfolio" sheetId="6" state="visible" r:id="rId6"/>
     <sheet name="Global Portfolio Map" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="Roadmap 0-18" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="Task 0 Checklist" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="Architecture" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Roadmap 0-18" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="Task 0 Checklist" sheetId="10" state="visible" r:id="rId10"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -198,6 +199,36 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>0</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="495300" cy="285750"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="1" name="Image 1" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
+</file>
+
+<file path=xl/drawings/drawing10.xml><?xml version="1.0" encoding="utf-8"?>
 <wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
@@ -1292,7 +1323,7 @@
       <c r="A1" s="1" t="n"/>
       <c r="B1" s="2" t="inlineStr">
         <is>
-          <t>PepsiCo Global Demand Forecasting — Project Overview</t>
+          <t>PepsiCo Demand Forecasting (Multi-Market) — Project Overview</t>
         </is>
       </c>
     </row>
@@ -1359,12 +1390,12 @@
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>Scaling approach</t>
+          <t>Architecture approach</t>
         </is>
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>One GLOBAL model with market x brand x category x store embeddings; transfers learning across geos and cold-starts new-market / new-product launches.</t>
+          <t>Chosen by BACKTESTING, not assumed. Path: local baselines -&gt; global multi-series model with market/retailer/store/brand/SKU embeddings -&gt; per-market comparison -&gt; hybrid refinement (segmented globals e.g. Beverages vs Snacks, optional geo fine-tuning, hierarchical reconciliation). A global model is NOT assumed to beat local. See the 'Architecture' sheet.</t>
         </is>
       </c>
     </row>
@@ -1449,6 +1480,228 @@
       <c r="B14" s="4" t="inlineStr">
         <is>
           <t>Independent learning project; NOT affiliated with or endorsed by PepsiCo. Generated brand tiles are stylized originals; logo/infographic are user-supplied. All trademarks belong to their owners.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="B1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B17"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="72" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="34" customHeight="1">
+      <c r="A1" s="1" t="n"/>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>Task 0 — Deliverables Checklist</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="22" customHeight="1">
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t>Deliverable</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="7" t="inlineStr">
+        <is>
+          <t>src/ layout package (cpg_forecast) installed editable</t>
+        </is>
+      </c>
+      <c r="B3" s="7" t="inlineStr">
+        <is>
+          <t>Done ✅</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="7" t="inlineStr">
+        <is>
+          <t>Python 3.12 virtual environment</t>
+        </is>
+      </c>
+      <c r="B4" s="7" t="inlineStr">
+        <is>
+          <t>Done ✅</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="7" t="inlineStr">
+        <is>
+          <t>pyproject.toml with dev + docs extras</t>
+        </is>
+      </c>
+      <c r="B5" s="7" t="inlineStr">
+        <is>
+          <t>Done ✅</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="7" t="inlineStr">
+        <is>
+          <t>ruff + black wired via pre-commit</t>
+        </is>
+      </c>
+      <c r="B6" s="7" t="inlineStr">
+        <is>
+          <t>Done ✅</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="7" t="inlineStr">
+        <is>
+          <t>Passing smoke tests (pytest)</t>
+        </is>
+      </c>
+      <c r="B7" s="7" t="inlineStr">
+        <is>
+          <t>Done ✅</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="7" t="inlineStr">
+        <is>
+          <t>Makefile (setup/lint/format/test/summary)</t>
+        </is>
+      </c>
+      <c r="B8" s="7" t="inlineStr">
+        <is>
+          <t>Done ✅</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="7" t="inlineStr">
+        <is>
+          <t>.gitignore + DVC-ready data/model folders</t>
+        </is>
+      </c>
+      <c r="B9" s="7" t="inlineStr">
+        <is>
+          <t>Done ✅</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="7" t="inlineStr">
+        <is>
+          <t>README with full roadmap + MIT LICENSE</t>
+        </is>
+      </c>
+      <c r="B10" s="7" t="inlineStr">
+        <is>
+          <t>Done ✅</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="7" t="inlineStr">
+        <is>
+          <t>Personal (non-Apple) git identity</t>
+        </is>
+      </c>
+      <c r="B11" s="7" t="inlineStr">
+        <is>
+          <t>Done ✅</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="7" t="inlineStr">
+        <is>
+          <t>Repo created &amp; pushed to personal GitHub</t>
+        </is>
+      </c>
+      <c r="B12" s="7" t="inlineStr">
+        <is>
+          <t>Done ✅</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="7" t="inlineStr">
+        <is>
+          <t>PepsiCo branding: real logo + generated brand icons</t>
+        </is>
+      </c>
+      <c r="B13" s="7" t="inlineStr">
+        <is>
+          <t>Done ✅</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="7" t="inlineStr">
+        <is>
+          <t>Multi-geo, multi-brand scope defined (matrix + portfolio)</t>
+        </is>
+      </c>
+      <c r="B14" s="7" t="inlineStr">
+        <is>
+          <t>Done ✅</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="7" t="inlineStr">
+        <is>
+          <t>Architecture framing: Local -&gt; Global -&gt; compare -&gt; Hybrid (evidence-driven)</t>
+        </is>
+      </c>
+      <c r="B15" s="7" t="inlineStr">
+        <is>
+          <t>Done ✅</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="7" t="inlineStr">
+        <is>
+          <t>Data residency documented (learning vs production)</t>
+        </is>
+      </c>
+      <c r="B16" s="7" t="inlineStr">
+        <is>
+          <t>Done ✅</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="7" t="inlineStr">
+        <is>
+          <t>Business + developer summary workbook (this file)</t>
+        </is>
+      </c>
+      <c r="B17" s="7" t="inlineStr">
+        <is>
+          <t>Done ✅</t>
         </is>
       </c>
     </row>
@@ -1661,12 +1914,12 @@
       </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>One GLOBAL deep-learning model with market/brand/category embeddings, forecasting SKU x store x day demand with uncertainty, feeding replenishment, DSD, production and promo planning.</t>
+          <t>A forecasting system selected EMPIRICALLY: local baselines first, then a global multi-series model with market/brand/store embeddings, compared per market, then hybrid refinement (segmented globals, optional geo fine-tuning, hierarchical reconciliation) adopted only where it beats the baselines.</t>
         </is>
       </c>
       <c r="C12" s="4" t="inlineStr">
         <is>
-          <t>Learns shared patterns across markets while respecting local behavior; scales to new geos.</t>
+          <t>Shares patterns where useful and localizes where needed — proven by backtests, not assumed.</t>
         </is>
       </c>
     </row>
@@ -1700,7 +1953,7 @@
       </c>
       <c r="C14" s="4" t="inlineStr">
         <is>
-          <t>De-risks the global rollout before any modeling.</t>
+          <t>De-risks the multi-market rollout before any modeling.</t>
         </is>
       </c>
     </row>
@@ -2187,7 +2440,7 @@
       </c>
       <c r="C13" s="4" t="inlineStr">
         <is>
-          <t>Seeds the embeddings that let one model scale across geos.</t>
+          <t>Seeds the embeddings that let models share signal across geos where it helps.</t>
         </is>
       </c>
     </row>
@@ -2907,6 +3160,207 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:C11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="26" customWidth="1" min="1" max="1"/>
+    <col width="62" customWidth="1" min="2" max="2"/>
+    <col width="46" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="34" customHeight="1">
+      <c r="A1" s="1" t="n"/>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>Architecture — Local vs Global vs Hybrid (evidence-driven)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="22" customHeight="1">
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t>Layer / Topic</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>What it is</t>
+        </is>
+      </c>
+      <c r="C2" s="3" t="inlineStr">
+        <is>
+          <t>Role / decision</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>Local baselines</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>One model per series/market (naive, seasonal-naive, ETS/ARIMA, LightGBM per group).</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>The BAR every deep model must beat, measured per market. Built in Task 4.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>Global multi-series model</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>One shared network trained across all series, conditioned on market/retailer/store/brand/category/SKU embeddings + local covariates (price, promo, calendar, weather).</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>Shares response shapes and enables cold-start for new SKUs/stores/markets. Built Tasks 5-9.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>Segmented global models</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>Separate global models per natural cluster — e.g. Beverages vs Snacks (very different dynamics), and/or per region.</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>Used where one pooled model shows negative transfer. Explored in Task 12.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>Geography fine-tuning / adapters</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>Global pre-train, then light per-market fine-tuning or adapter layers.</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>Optional refinement for large markets that deviate from the shared pattern.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>Hierarchical reconciliation</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>Make SKU x store forecasts coherent with store/brand/category/geography totals (bottom-up / MinT).</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>Applied on top of the chosen model so all levels agree.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>How the architecture is chosen</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>Market-level rolling-origin backtesting on WRMSSE + interval calibration decides how much pooling actually helps.</t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="inlineStr">
+        <is>
+          <t>Architecture is a RESULT, not an assumption. A global model is NOT assumed to outperform local.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>Data residency — this learning project</t>
+        </is>
+      </c>
+      <c r="B10" s="4" t="inlineStr">
+        <is>
+          <t>Cross-border pooling is ALLOWED: we use the public M5 (Walmart) proxy dataset, not real PepsiCo country data.</t>
+        </is>
+      </c>
+      <c r="C10" s="4" t="inlineStr">
+        <is>
+          <t>Optimize for understanding the modeling concepts first.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>Data residency — production constraint</t>
+        </is>
+      </c>
+      <c r="B11" s="4" t="inlineStr">
+        <is>
+          <t>In a real PepsiCo deployment, raw data may be legally required to stay within region/country boundaries (e.g. India DPDP Act).</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="inlineStr">
+        <is>
+          <t>Then use region-segmented global models, local fine-tuning, or federated learning depending on legal requirements.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="B1:C1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:E21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -3068,17 +3522,17 @@
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>Classical baselines &amp; eval harness</t>
+          <t>Local baselines &amp; eval harness</t>
         </is>
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>why baselines matter</t>
+          <t>local per-series/market baselines = the bar to beat</t>
         </is>
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t>WRMSSE, backtesting, tracking</t>
+          <t>WRMSSE, market-level backtesting, tracking</t>
         </is>
       </c>
       <c r="E7" s="4" t="inlineStr">
@@ -3203,17 +3657,17 @@
       </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>Transformer / TFT</t>
+          <t>Transformer / TFT (global model)</t>
         </is>
       </c>
       <c r="C12" s="4" t="inlineStr">
         <is>
-          <t>self-attention, static covariates (geo/brand)</t>
+          <t>self-attention + entity embeddings; global vs local per market</t>
         </is>
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
-          <t>large-model training</t>
+          <t>large-model training, market-level comparison</t>
         </is>
       </c>
       <c r="E12" s="4" t="inlineStr">
@@ -3284,17 +3738,17 @@
       </c>
       <c r="B15" s="4" t="inlineStr">
         <is>
-          <t>Cloud full-scale training</t>
+          <t>Cloud training + hybrid refinement</t>
         </is>
       </c>
       <c r="C15" s="4" t="inlineStr">
         <is>
-          <t>global model across all markets</t>
+          <t>segmented globals, geo fine-tuning, reconciliation</t>
         </is>
       </c>
       <c r="D15" s="4" t="inlineStr">
         <is>
-          <t>training-as-code</t>
+          <t>training-as-code, architecture chosen by backtest</t>
         </is>
       </c>
       <c r="E15" s="4" t="inlineStr">
@@ -3472,202 +3926,4 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:B15"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="65" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="34" customHeight="1">
-      <c r="A1" s="1" t="n"/>
-      <c r="B1" s="2" t="inlineStr">
-        <is>
-          <t>Task 0 — Deliverables Checklist</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="22" customHeight="1">
-      <c r="A2" s="3" t="inlineStr">
-        <is>
-          <t>Deliverable</t>
-        </is>
-      </c>
-      <c r="B2" s="3" t="inlineStr">
-        <is>
-          <t>Status</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="7" t="inlineStr">
-        <is>
-          <t>src/ layout package (cpg_forecast) installed editable</t>
-        </is>
-      </c>
-      <c r="B3" s="7" t="inlineStr">
-        <is>
-          <t>Done ✅</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="7" t="inlineStr">
-        <is>
-          <t>Python 3.12 virtual environment</t>
-        </is>
-      </c>
-      <c r="B4" s="7" t="inlineStr">
-        <is>
-          <t>Done ✅</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="7" t="inlineStr">
-        <is>
-          <t>pyproject.toml with dev + docs extras</t>
-        </is>
-      </c>
-      <c r="B5" s="7" t="inlineStr">
-        <is>
-          <t>Done ✅</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="7" t="inlineStr">
-        <is>
-          <t>ruff + black wired via pre-commit</t>
-        </is>
-      </c>
-      <c r="B6" s="7" t="inlineStr">
-        <is>
-          <t>Done ✅</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="7" t="inlineStr">
-        <is>
-          <t>Passing smoke tests (pytest)</t>
-        </is>
-      </c>
-      <c r="B7" s="7" t="inlineStr">
-        <is>
-          <t>Done ✅</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="7" t="inlineStr">
-        <is>
-          <t>Makefile (setup/lint/format/test/summary)</t>
-        </is>
-      </c>
-      <c r="B8" s="7" t="inlineStr">
-        <is>
-          <t>Done ✅</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="7" t="inlineStr">
-        <is>
-          <t>.gitignore + DVC-ready data/model folders</t>
-        </is>
-      </c>
-      <c r="B9" s="7" t="inlineStr">
-        <is>
-          <t>Done ✅</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="7" t="inlineStr">
-        <is>
-          <t>README with full roadmap + MIT LICENSE</t>
-        </is>
-      </c>
-      <c r="B10" s="7" t="inlineStr">
-        <is>
-          <t>Done ✅</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="7" t="inlineStr">
-        <is>
-          <t>Personal (non-Apple) git identity</t>
-        </is>
-      </c>
-      <c r="B11" s="7" t="inlineStr">
-        <is>
-          <t>Done ✅</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="7" t="inlineStr">
-        <is>
-          <t>Repo created &amp; pushed to personal GitHub</t>
-        </is>
-      </c>
-      <c r="B12" s="7" t="inlineStr">
-        <is>
-          <t>Done ✅</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="7" t="inlineStr">
-        <is>
-          <t>PepsiCo branding: real logo + generated brand icons</t>
-        </is>
-      </c>
-      <c r="B13" s="7" t="inlineStr">
-        <is>
-          <t>Done ✅</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="7" t="inlineStr">
-        <is>
-          <t>Multi-geo, multi-brand scope defined (matrix + portfolio)</t>
-        </is>
-      </c>
-      <c r="B14" s="7" t="inlineStr">
-        <is>
-          <t>Done ✅</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="7" t="inlineStr">
-        <is>
-          <t>Business + developer summary workbook (this file)</t>
-        </is>
-      </c>
-      <c r="B15" s="7" t="inlineStr">
-        <is>
-          <t>Done ✅</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="B1"/>
-  </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
-</worksheet>
 </file>
</xml_diff>